<commit_message>
problem: check if a LL is a palindrome
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
   <si>
     <t>date</t>
   </si>
@@ -175,6 +175,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/longest-palindromic-substring/description/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check if a LL is a palindrome</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/palindrome-linked-list/</t>
   </si>
 </sst>
 </file>
@@ -998,7 +1004,7 @@
       </c>
     </row>
     <row r="26" ht="14.25">
-      <c r="A26" s="3">
+      <c r="A26" s="1">
         <v>46056</v>
       </c>
       <c r="B26" t="s">
@@ -1006,6 +1012,17 @@
       </c>
       <c r="C26" s="2" t="s">
         <v>52</v>
+      </c>
+    </row>
+    <row r="27" ht="14.25">
+      <c r="A27" s="3">
+        <v>46084</v>
+      </c>
+      <c r="B27" t="s">
+        <v>53</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1034,6 +1051,7 @@
     <hyperlink r:id="rId22" ref="C24"/>
     <hyperlink r:id="rId23" ref="C25"/>
     <hyperlink r:id="rId24" ref="C26"/>
+    <hyperlink r:id="rId25" ref="C27"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
problem : clone graph
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
   <si>
     <t>date</t>
   </si>
@@ -289,6 +289,12 @@
   </si>
   <si>
     <t>https://leetcode.com/contest/weekly-contest-492/problems/minimum-cost-to-partition-a-binary-string/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">clone graph</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/clone-graph/</t>
   </si>
 </sst>
 </file>
@@ -329,13 +335,14 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1312,6 +1319,9 @@
       </c>
     </row>
     <row r="44" ht="14.25">
+      <c r="A44" s="4">
+        <v>46089</v>
+      </c>
       <c r="B44" t="s">
         <v>87</v>
       </c>
@@ -1320,11 +1330,25 @@
       </c>
     </row>
     <row r="45" ht="14.25">
+      <c r="A45" s="4">
+        <v>46089</v>
+      </c>
       <c r="B45" t="s">
         <v>89</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>90</v>
+      </c>
+    </row>
+    <row r="46" ht="14.25">
+      <c r="A46" s="4">
+        <v>46089</v>
+      </c>
+      <c r="B46" t="s">
+        <v>91</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -1372,6 +1396,7 @@
     <hyperlink r:id="rId41" ref="C43"/>
     <hyperlink r:id="rId42" ref="C44"/>
     <hyperlink r:id="rId43" ref="C45"/>
+    <hyperlink r:id="rId44" ref="C46"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
problem: course schedule II
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
   <si>
     <t>date</t>
   </si>
@@ -324,7 +324,13 @@
     <t xml:space="preserve">course schedule</t>
   </si>
   <si>
-    <t>https://leetcode.com/problems/course-schedule/description/?envType=study-plan-v2&amp;envId=top-interview-150</t>
+    <t>https://leetcode.com/problems/course-schedule/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">course schedule II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/course-schedule-ii/</t>
   </si>
 </sst>
 </file>
@@ -365,14 +371,13 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1393,7 +1398,7 @@
       </c>
     </row>
     <row r="48" ht="14.25">
-      <c r="A48" s="4">
+      <c r="A48" s="1">
         <v>46090</v>
       </c>
       <c r="B48" t="s">
@@ -1404,7 +1409,7 @@
       </c>
     </row>
     <row r="49" ht="14.25">
-      <c r="A49" s="4">
+      <c r="A49" s="1">
         <v>46091</v>
       </c>
       <c r="B49" t="s">
@@ -1415,7 +1420,7 @@
       </c>
     </row>
     <row r="50" ht="14.25">
-      <c r="A50" s="4">
+      <c r="A50" s="1">
         <v>46091</v>
       </c>
       <c r="B50" t="s">
@@ -1426,7 +1431,7 @@
       </c>
     </row>
     <row r="51" ht="14.25">
-      <c r="A51" s="4">
+      <c r="A51" s="1">
         <v>46091</v>
       </c>
       <c r="B51" t="s">
@@ -1437,7 +1442,15 @@
       </c>
     </row>
     <row r="52" ht="14.25">
-      <c r="A52" s="4"/>
+      <c r="A52" s="1">
+        <v>46092</v>
+      </c>
+      <c r="B52" t="s">
+        <v>103</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>104</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1490,6 +1503,7 @@
     <hyperlink r:id="rId47" ref="C49"/>
     <hyperlink r:id="rId48" ref="C50"/>
     <hyperlink r:id="rId49" ref="C51"/>
+    <hyperlink r:id="rId50" ref="C52"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
problem: min. genetic mutation.
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="109">
   <si>
     <t>date</t>
   </si>
@@ -337,6 +337,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/snakes-and-ladders/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum Genetic Mutation</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-genetic-mutation</t>
   </si>
 </sst>
 </file>
@@ -377,13 +383,14 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1459,11 +1466,25 @@
       </c>
     </row>
     <row r="53" ht="14.25">
+      <c r="A53" s="4">
+        <v>46093</v>
+      </c>
       <c r="B53" t="s">
         <v>105</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>106</v>
+      </c>
+    </row>
+    <row r="54" ht="14.25">
+      <c r="A54" s="4">
+        <v>46094</v>
+      </c>
+      <c r="B54" t="s">
+        <v>107</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -1519,6 +1540,7 @@
     <hyperlink r:id="rId49" ref="C51"/>
     <hyperlink r:id="rId50" ref="C52"/>
     <hyperlink r:id="rId51" ref="C53"/>
+    <hyperlink r:id="rId52" ref="C54"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Solved 2 related problems of monotonic stack: largest rectangle in histogram and maximal rectangle
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="131">
   <si>
     <t>date</t>
   </si>
@@ -397,6 +397,18 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/word-search/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">maximal rectangle</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/maximal-rectangle/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">largest rectangle in histogram</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/largest-rectangle-in-histogram/</t>
   </si>
 </sst>
 </file>
@@ -1630,7 +1642,7 @@
       </c>
     </row>
     <row r="63" ht="14.25">
-      <c r="A63" s="4">
+      <c r="A63" s="1">
         <v>46100</v>
       </c>
       <c r="B63" t="s">
@@ -1638,6 +1650,28 @@
       </c>
       <c r="C63" s="2" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="64" ht="14.25">
+      <c r="A64" s="4">
+        <v>46100</v>
+      </c>
+      <c r="B64" t="s">
+        <v>127</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="65" ht="14.25">
+      <c r="A65" s="4">
+        <v>46100</v>
+      </c>
+      <c r="B65" t="s">
+        <v>129</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -1703,6 +1737,8 @@
     <hyperlink r:id="rId59" ref="C61"/>
     <hyperlink r:id="rId60" ref="C62"/>
     <hyperlink r:id="rId61" ref="C63"/>
+    <hyperlink r:id="rId62" ref="C64"/>
+    <hyperlink r:id="rId63" ref="C65"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: find identical tree or not
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="135">
   <si>
     <t>date</t>
   </si>
@@ -415,6 +415,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/maximum-depth-of-binary-tree/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">same tree</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/same-tree/</t>
   </si>
 </sst>
 </file>
@@ -1681,7 +1687,7 @@
       </c>
     </row>
     <row r="66" ht="14.25">
-      <c r="A66" s="4">
+      <c r="A66" s="1">
         <v>46101</v>
       </c>
       <c r="B66" t="s">
@@ -1689,6 +1695,17 @@
       </c>
       <c r="C66" s="2" t="s">
         <v>132</v>
+      </c>
+    </row>
+    <row r="67" ht="14.25">
+      <c r="A67" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B67" t="s">
+        <v>133</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -1757,6 +1774,7 @@
     <hyperlink r:id="rId62" ref="C64"/>
     <hyperlink r:id="rId63" ref="C65"/>
     <hyperlink r:id="rId64" ref="C66"/>
+    <hyperlink r:id="rId65" ref="C67"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problems: Inorder, preorder and postorder using stack and morris traversals and flatten binary tree problem
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="153">
   <si>
     <t>date</t>
   </si>
@@ -451,6 +451,30 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/populating-next-right-pointers-in-each-node-ii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In order traversal</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/binary-tree-inorder-traversal/description/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre order traversal</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/binary-tree-preorder-traversal/description/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">post order traversal</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/binary-tree-postorder-traversal/description/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flatten binary tree to linked list</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/flatten-binary-tree-to-linked-list/</t>
   </si>
 </sst>
 </file>
@@ -1784,7 +1808,7 @@
       </c>
     </row>
     <row r="72" ht="14.25">
-      <c r="A72" s="5">
+      <c r="A72" s="1">
         <v>46104</v>
       </c>
       <c r="B72" t="s">
@@ -1792,6 +1816,50 @@
       </c>
       <c r="C72" s="2" t="s">
         <v>144</v>
+      </c>
+    </row>
+    <row r="73" ht="14.25">
+      <c r="A73" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B73" t="s">
+        <v>145</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="74" ht="14.25">
+      <c r="A74" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B74" t="s">
+        <v>147</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="75" ht="14.25">
+      <c r="A75" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B75" t="s">
+        <v>149</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="76" ht="14.25">
+      <c r="A76" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B76" t="s">
+        <v>151</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>152</v>
       </c>
     </row>
   </sheetData>
@@ -1866,6 +1934,10 @@
     <hyperlink r:id="rId68" ref="C70"/>
     <hyperlink r:id="rId69" ref="C71"/>
     <hyperlink r:id="rId70" ref="C72"/>
+    <hyperlink r:id="rId71" ref="C73"/>
+    <hyperlink r:id="rId72" ref="C74"/>
+    <hyperlink r:id="rId73" ref="C75"/>
+    <hyperlink r:id="rId74" ref="C76"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problems: BST Iterator and Binary Tree Max. Path Sum
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="163">
   <si>
     <t>date</t>
   </si>
@@ -493,6 +493,18 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/sum-root-to-leaf-numbers/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binary Tree Max Path Sum</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/binary-tree-maximum-path-sum/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BST Iterator</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/binary-search-tree-iterator/</t>
   </si>
 </sst>
 </file>
@@ -1881,7 +1893,7 @@
       </c>
     </row>
     <row r="77" ht="14.25">
-      <c r="A77" s="5">
+      <c r="A77" s="1">
         <v>46106</v>
       </c>
       <c r="B77" t="s">
@@ -1892,7 +1904,7 @@
       </c>
     </row>
     <row r="78" ht="14.25">
-      <c r="A78" s="5">
+      <c r="A78" s="1">
         <v>46106</v>
       </c>
       <c r="B78" t="s">
@@ -1903,7 +1915,7 @@
       </c>
     </row>
     <row r="79" ht="14.25">
-      <c r="A79" s="5">
+      <c r="A79" s="1">
         <v>46106</v>
       </c>
       <c r="B79" t="s">
@@ -1911,6 +1923,28 @@
       </c>
       <c r="C79" s="2" t="s">
         <v>158</v>
+      </c>
+    </row>
+    <row r="80" ht="14.25">
+      <c r="A80" s="1">
+        <v>46107</v>
+      </c>
+      <c r="B80" t="s">
+        <v>159</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="81" ht="14.25">
+      <c r="A81" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B81" t="s">
+        <v>161</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -1992,6 +2026,8 @@
     <hyperlink r:id="rId75" ref="C77"/>
     <hyperlink r:id="rId76" ref="C78"/>
     <hyperlink r:id="rId77" ref="C79"/>
+    <hyperlink r:id="rId78" ref="C80"/>
+    <hyperlink r:id="rId79" ref="C81"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: count complete tree nodes
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
   <si>
     <t>date</t>
   </si>
@@ -505,6 +505,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/binary-search-tree-iterator/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Count complete tree nodes </t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/count-complete-tree-nodes/</t>
   </si>
 </sst>
 </file>
@@ -1937,7 +1943,7 @@
       </c>
     </row>
     <row r="81" ht="14.25">
-      <c r="A81" s="5">
+      <c r="A81" s="1">
         <v>46107</v>
       </c>
       <c r="B81" t="s">
@@ -1945,6 +1951,17 @@
       </c>
       <c r="C81" s="2" t="s">
         <v>162</v>
+      </c>
+    </row>
+    <row r="82" ht="14.25">
+      <c r="A82" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B82" t="s">
+        <v>163</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -2028,6 +2045,7 @@
     <hyperlink r:id="rId77" ref="C79"/>
     <hyperlink r:id="rId78" ref="C80"/>
     <hyperlink r:id="rId79" ref="C81"/>
+    <hyperlink r:id="rId80" ref="C82"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: LCA of binary tree
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="167">
   <si>
     <t>date</t>
   </si>
@@ -511,6 +511,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/count-complete-tree-nodes/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LCA of Binary Tree</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-tree/</t>
   </si>
 </sst>
 </file>
@@ -1954,7 +1960,7 @@
       </c>
     </row>
     <row r="82" ht="14.25">
-      <c r="A82" s="5">
+      <c r="A82" s="1">
         <v>46107</v>
       </c>
       <c r="B82" t="s">
@@ -1962,6 +1968,17 @@
       </c>
       <c r="C82" s="2" t="s">
         <v>164</v>
+      </c>
+    </row>
+    <row r="83" ht="14.25">
+      <c r="A83" s="5">
+        <v>46108</v>
+      </c>
+      <c r="B83" t="s">
+        <v>165</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -2046,6 +2063,7 @@
     <hyperlink r:id="rId78" ref="C80"/>
     <hyperlink r:id="rId79" ref="C81"/>
     <hyperlink r:id="rId80" ref="C82"/>
+    <hyperlink r:id="rId81" ref="C83"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: single number II
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="201">
   <si>
     <t>date</t>
   </si>
@@ -613,6 +613,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/number-of-1-bits/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Single Number II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/single-number-ii/</t>
   </si>
 </sst>
 </file>
@@ -2232,7 +2238,7 @@
       </c>
     </row>
     <row r="98" ht="14.25">
-      <c r="A98" s="5">
+      <c r="A98" s="1">
         <v>46113</v>
       </c>
       <c r="B98" t="s">
@@ -2243,7 +2249,7 @@
       </c>
     </row>
     <row r="99" ht="14.25">
-      <c r="A99" s="5">
+      <c r="A99" s="1">
         <v>46113</v>
       </c>
       <c r="B99" t="s">
@@ -2251,6 +2257,17 @@
       </c>
       <c r="C99" s="2" t="s">
         <v>198</v>
+      </c>
+    </row>
+    <row r="100" ht="14.25">
+      <c r="A100" s="5">
+        <v>46114</v>
+      </c>
+      <c r="B100" t="s">
+        <v>199</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -2352,6 +2369,7 @@
     <hyperlink r:id="rId95" ref="C97"/>
     <hyperlink r:id="rId96" ref="C98"/>
     <hyperlink r:id="rId97" ref="C99"/>
+    <hyperlink r:id="rId98" ref="C100"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: max. product sub-array
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="209">
   <si>
     <t>date</t>
   </si>
@@ -637,6 +637,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/ipo/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max product subarray</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/maximum-product-subarray/</t>
   </si>
 </sst>
 </file>
@@ -2311,7 +2317,7 @@
       </c>
     </row>
     <row r="103" ht="14.25">
-      <c r="A103" s="5">
+      <c r="A103" s="1">
         <v>46115</v>
       </c>
       <c r="B103" t="s">
@@ -2319,6 +2325,17 @@
       </c>
       <c r="C103" s="2" t="s">
         <v>206</v>
+      </c>
+    </row>
+    <row r="104" ht="14.25">
+      <c r="A104" s="5">
+        <v>46115</v>
+      </c>
+      <c r="B104" t="s">
+        <v>207</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -2424,6 +2441,7 @@
     <hyperlink r:id="rId99" ref="C101"/>
     <hyperlink r:id="rId100" ref="C102"/>
     <hyperlink r:id="rId101" ref="C103"/>
+    <hyperlink r:id="rId102" ref="C104"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: find k pairs with smallest sums
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="211">
   <si>
     <t>date</t>
   </si>
@@ -643,6 +643,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/maximum-product-subarray/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">find k pairs with smallest sums</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/find-k-pairs-with-smallest-sums/</t>
   </si>
 </sst>
 </file>
@@ -2328,7 +2334,7 @@
       </c>
     </row>
     <row r="104" ht="14.25">
-      <c r="A104" s="5">
+      <c r="A104" s="1">
         <v>46115</v>
       </c>
       <c r="B104" t="s">
@@ -2336,6 +2342,17 @@
       </c>
       <c r="C104" s="2" t="s">
         <v>208</v>
+      </c>
+    </row>
+    <row r="105" ht="14.25">
+      <c r="A105" s="5">
+        <v>46115</v>
+      </c>
+      <c r="B105" t="s">
+        <v>209</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>210</v>
       </c>
     </row>
   </sheetData>
@@ -2442,6 +2459,7 @@
     <hyperlink r:id="rId100" ref="C102"/>
     <hyperlink r:id="rId101" ref="C103"/>
     <hyperlink r:id="rId102" ref="C104"/>
+    <hyperlink r:id="rId103" ref="C105"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: find median of data stream
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="213">
   <si>
     <t>date</t>
   </si>
@@ -649,6 +649,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/find-k-pairs-with-smallest-sums/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">find median from data stream</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/find-median-from-data-stream/</t>
   </si>
 </sst>
 </file>
@@ -2345,7 +2351,7 @@
       </c>
     </row>
     <row r="105" ht="14.25">
-      <c r="A105" s="5">
+      <c r="A105" s="1">
         <v>46115</v>
       </c>
       <c r="B105" t="s">
@@ -2353,6 +2359,17 @@
       </c>
       <c r="C105" s="2" t="s">
         <v>210</v>
+      </c>
+    </row>
+    <row r="106" ht="14.25">
+      <c r="A106" s="5">
+        <v>46116</v>
+      </c>
+      <c r="B106" t="s">
+        <v>211</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -2460,6 +2477,7 @@
     <hyperlink r:id="rId101" ref="C103"/>
     <hyperlink r:id="rId102" ref="C104"/>
     <hyperlink r:id="rId103" ref="C105"/>
+    <hyperlink r:id="rId104" ref="C106"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problems: peak element Binary Search and Prefix sum range query
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="221">
   <si>
     <t>date</t>
   </si>
@@ -667,6 +667,18 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/search-a-2d-matrix/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">find peak element</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/find-peak-element/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prefix sum range query</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/prefix-sum-range-query/1</t>
   </si>
 </sst>
 </file>
@@ -2396,7 +2408,7 @@
       </c>
     </row>
     <row r="108" ht="14.25">
-      <c r="A108" s="5">
+      <c r="A108" s="1">
         <v>46117</v>
       </c>
       <c r="B108" t="s">
@@ -2404,6 +2416,28 @@
       </c>
       <c r="C108" s="2" t="s">
         <v>216</v>
+      </c>
+    </row>
+    <row r="109" ht="14.25">
+      <c r="A109" s="5">
+        <v>46118</v>
+      </c>
+      <c r="B109" t="s">
+        <v>217</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="110" ht="14.25">
+      <c r="A110" s="5">
+        <v>46118</v>
+      </c>
+      <c r="B110" t="s">
+        <v>219</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>220</v>
       </c>
     </row>
   </sheetData>
@@ -2514,6 +2548,8 @@
     <hyperlink r:id="rId104" ref="C106"/>
     <hyperlink r:id="rId105" ref="C107"/>
     <hyperlink r:id="rId106" ref="C108"/>
+    <hyperlink r:id="rId107" ref="C109"/>
+    <hyperlink r:id="rId108" ref="C110"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: design circular queue
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="237">
   <si>
     <t>date</t>
   </si>
@@ -721,6 +721,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/find-minimum-in-rotated-sorted-array/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">design circular queue</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/design-circular-queue/</t>
   </si>
 </sst>
 </file>
@@ -2549,7 +2555,7 @@
       </c>
     </row>
     <row r="117" ht="14.25">
-      <c r="A117" s="5">
+      <c r="A117" s="1">
         <v>46120</v>
       </c>
       <c r="B117" t="s">
@@ -2557,6 +2563,17 @@
       </c>
       <c r="C117" s="2" t="s">
         <v>234</v>
+      </c>
+    </row>
+    <row r="118" ht="14.25">
+      <c r="A118" s="5">
+        <v>46120</v>
+      </c>
+      <c r="B118" t="s">
+        <v>235</v>
+      </c>
+      <c r="C118" s="2" t="s">
+        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -2676,6 +2693,7 @@
     <hyperlink r:id="rId113" ref="C115"/>
     <hyperlink r:id="rId114" ref="C116"/>
     <hyperlink r:id="rId115" ref="C117"/>
+    <hyperlink r:id="rId116" ref="C118"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: max. subArray sum
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="243">
   <si>
     <t>date</t>
   </si>
@@ -739,6 +739,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/median-of-two-sorted-arrays/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">maximum subarray</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/maximum-subarray</t>
   </si>
 </sst>
 </file>
@@ -2600,7 +2606,7 @@
       </c>
     </row>
     <row r="120" ht="14.25">
-      <c r="A120" s="5">
+      <c r="A120" s="1">
         <v>46121</v>
       </c>
       <c r="B120" t="s">
@@ -2608,6 +2614,17 @@
       </c>
       <c r="C120" s="2" t="s">
         <v>240</v>
+      </c>
+    </row>
+    <row r="121" ht="14.25">
+      <c r="A121" s="5">
+        <v>46122</v>
+      </c>
+      <c r="B121" t="s">
+        <v>241</v>
+      </c>
+      <c r="C121" s="2" t="s">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -2730,6 +2747,7 @@
     <hyperlink r:id="rId116" ref="C118"/>
     <hyperlink r:id="rId117" ref="C119"/>
     <hyperlink r:id="rId118" ref="C120"/>
+    <hyperlink r:id="rId119" ref="C121"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem : sort 2 LL using Merge Sort
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="249">
   <si>
     <t>date</t>
   </si>
@@ -757,6 +757,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/convert-sorted-array-to-binary-search-tree/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sort List</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/sort-list/</t>
   </si>
 </sst>
 </file>
@@ -2654,7 +2660,7 @@
       </c>
     </row>
     <row r="123" ht="14.25">
-      <c r="A123" s="6">
+      <c r="A123" s="1">
         <v>46123</v>
       </c>
       <c r="B123" t="s">
@@ -2662,6 +2668,17 @@
       </c>
       <c r="C123" s="2" t="s">
         <v>246</v>
+      </c>
+    </row>
+    <row r="124" ht="14.25">
+      <c r="A124" s="6">
+        <v>46124</v>
+      </c>
+      <c r="B124" t="s">
+        <v>247</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>248</v>
       </c>
     </row>
   </sheetData>
@@ -2787,6 +2804,7 @@
     <hyperlink r:id="rId119" ref="C121"/>
     <hyperlink r:id="rId120" ref="C122"/>
     <hyperlink r:id="rId121" ref="C123"/>
+    <hyperlink r:id="rId122" ref="C124"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: reverse ll II
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="261">
   <si>
     <t>date</t>
   </si>
@@ -793,6 +793,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/copy-list-with-random-pointer/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reverse linked list II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/reverse-linked-list-ii/</t>
   </si>
 </sst>
 </file>
@@ -2756,7 +2762,7 @@
       </c>
     </row>
     <row r="129" ht="14.25">
-      <c r="A129" s="6">
+      <c r="A129" s="1">
         <v>46130</v>
       </c>
       <c r="B129" t="s">
@@ -2764,6 +2770,17 @@
       </c>
       <c r="C129" s="2" t="s">
         <v>258</v>
+      </c>
+    </row>
+    <row r="130" ht="14.25">
+      <c r="A130" s="6">
+        <v>46130</v>
+      </c>
+      <c r="B130" t="s">
+        <v>259</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>260</v>
       </c>
     </row>
   </sheetData>
@@ -2895,6 +2912,7 @@
     <hyperlink r:id="rId125" ref="C127"/>
     <hyperlink r:id="rId126" ref="C128"/>
     <hyperlink r:id="rId127" ref="C129"/>
+    <hyperlink r:id="rId128" ref="C130"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: reverse nodes in k grp
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="263">
   <si>
     <t>date</t>
   </si>
@@ -799,6 +799,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/reverse-linked-list-ii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reverse nodes in k grp</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/reverse-nodes-in-k-group/</t>
   </si>
 </sst>
 </file>
@@ -2773,7 +2779,7 @@
       </c>
     </row>
     <row r="130" ht="14.25">
-      <c r="A130" s="6">
+      <c r="A130" s="1">
         <v>46130</v>
       </c>
       <c r="B130" t="s">
@@ -2781,6 +2787,17 @@
       </c>
       <c r="C130" s="2" t="s">
         <v>260</v>
+      </c>
+    </row>
+    <row r="131" ht="14.25">
+      <c r="A131" s="6">
+        <v>46131</v>
+      </c>
+      <c r="B131" t="s">
+        <v>261</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -2913,6 +2930,7 @@
     <hyperlink r:id="rId126" ref="C128"/>
     <hyperlink r:id="rId127" ref="C129"/>
     <hyperlink r:id="rId128" ref="C130"/>
+    <hyperlink r:id="rId129" ref="C131"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: remove duplicates from sorted list and rotate list
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="267">
   <si>
     <t>date</t>
   </si>
@@ -805,6 +805,18 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/reverse-nodes-in-k-group/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">remove duplicates from sorted list II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/remove-duplicates-from-sorted-list-ii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rotate list</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/rotate-list/</t>
   </si>
 </sst>
 </file>
@@ -2790,7 +2802,7 @@
       </c>
     </row>
     <row r="131" ht="14.25">
-      <c r="A131" s="6">
+      <c r="A131" s="1">
         <v>46131</v>
       </c>
       <c r="B131" t="s">
@@ -2798,6 +2810,28 @@
       </c>
       <c r="C131" s="2" t="s">
         <v>262</v>
+      </c>
+    </row>
+    <row r="132" ht="14.25">
+      <c r="A132" s="6">
+        <v>46132</v>
+      </c>
+      <c r="B132" t="s">
+        <v>263</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="133" ht="14.25">
+      <c r="A133" s="6">
+        <v>46132</v>
+      </c>
+      <c r="B133" t="s">
+        <v>265</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -2931,6 +2965,8 @@
     <hyperlink r:id="rId127" ref="C129"/>
     <hyperlink r:id="rId128" ref="C130"/>
     <hyperlink r:id="rId129" ref="C131"/>
+    <hyperlink r:id="rId130" ref="C132"/>
+    <hyperlink r:id="rId131" ref="C133"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: evaluate reverse polish notation
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="275">
   <si>
     <t>date</t>
   </si>
@@ -835,6 +835,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/min-stack/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">evaluate reverse polish notation</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/evaluate-reverse-polish-notation/</t>
   </si>
 </sst>
 </file>
@@ -2875,7 +2881,7 @@
       </c>
     </row>
     <row r="136" ht="14.25">
-      <c r="A136" s="6">
+      <c r="A136" s="1">
         <v>46134</v>
       </c>
       <c r="B136" t="s">
@@ -2883,6 +2889,17 @@
       </c>
       <c r="C136" s="2" t="s">
         <v>272</v>
+      </c>
+    </row>
+    <row r="137" ht="14.25">
+      <c r="A137" s="6">
+        <v>46134</v>
+      </c>
+      <c r="B137" t="s">
+        <v>273</v>
+      </c>
+      <c r="C137" s="2" t="s">
+        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -3021,6 +3038,7 @@
     <hyperlink r:id="rId132" ref="C134"/>
     <hyperlink r:id="rId133" ref="C135"/>
     <hyperlink r:id="rId134" ref="C136"/>
+    <hyperlink r:id="rId135" ref="C137"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: set matrix zeroes
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="311">
   <si>
     <t>date</t>
   </si>
@@ -943,6 +943,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/rotate-image/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">set matrix zeroes</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/set-matrix-zeroes/</t>
   </si>
 </sst>
 </file>
@@ -3190,6 +3196,17 @@
         <v>308</v>
       </c>
     </row>
+    <row r="155" ht="14.25">
+      <c r="A155" s="1">
+        <v>46148</v>
+      </c>
+      <c r="B155" t="s">
+        <v>309</v>
+      </c>
+      <c r="C155" s="2" t="s">
+        <v>310</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3344,6 +3361,7 @@
     <hyperlink r:id="rId150" ref="C152"/>
     <hyperlink r:id="rId151" ref="C153"/>
     <hyperlink r:id="rId152" ref="C154"/>
+    <hyperlink r:id="rId153" ref="C155"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: game of life
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="313">
   <si>
     <t>date</t>
   </si>
@@ -949,6 +949,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/set-matrix-zeroes/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min. size subarray sum</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-size-subarray-sum/</t>
   </si>
 </sst>
 </file>
@@ -3207,6 +3213,17 @@
         <v>310</v>
       </c>
     </row>
+    <row r="156" ht="14.25">
+      <c r="A156" s="1">
+        <v>46149</v>
+      </c>
+      <c r="B156" t="s">
+        <v>311</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>312</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3362,6 +3379,7 @@
     <hyperlink r:id="rId151" ref="C153"/>
     <hyperlink r:id="rId152" ref="C154"/>
     <hyperlink r:id="rId153" ref="C155"/>
+    <hyperlink r:id="rId154" ref="C156"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: longest substring without repeating chars
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="317">
   <si>
     <t>date</t>
   </si>
@@ -955,6 +955,18 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/minimum-size-subarray-sum/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">game of life</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/game-of-life/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">longest substring without repeating character</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/longest-substring-without-repeating-characters/</t>
   </si>
 </sst>
 </file>
@@ -3225,7 +3237,26 @@
       </c>
     </row>
     <row r="157" ht="14.25">
-      <c r="A157" s="1"/>
+      <c r="A157" s="1">
+        <v>46149</v>
+      </c>
+      <c r="B157" t="s">
+        <v>313</v>
+      </c>
+      <c r="C157" s="2" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="158" ht="14.25">
+      <c r="A158" s="1">
+        <v>46149</v>
+      </c>
+      <c r="B158" t="s">
+        <v>315</v>
+      </c>
+      <c r="C158" s="2" t="s">
+        <v>316</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3383,6 +3414,8 @@
     <hyperlink r:id="rId152" ref="C154"/>
     <hyperlink r:id="rId153" ref="C155"/>
     <hyperlink r:id="rId154" ref="C156"/>
+    <hyperlink r:id="rId155" ref="C157"/>
+    <hyperlink r:id="rId156" ref="C158"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: remove duplicates from sorted array II
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="341">
   <si>
     <t>date</t>
   </si>
@@ -1033,6 +1033,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">remove duplicates from sorted array II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array-ii/</t>
   </si>
 </sst>
 </file>
@@ -3445,6 +3451,17 @@
         <v>338</v>
       </c>
     </row>
+    <row r="170" ht="14.25">
+      <c r="A170" s="1">
+        <v>46154</v>
+      </c>
+      <c r="B170" t="s">
+        <v>339</v>
+      </c>
+      <c r="C170" s="2" t="s">
+        <v>340</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3614,6 +3631,7 @@
     <hyperlink r:id="rId165" ref="C167"/>
     <hyperlink r:id="rId166" ref="C168"/>
     <hyperlink r:id="rId167" ref="C169"/>
+    <hyperlink r:id="rId168" ref="C170"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problems: reverse words in a string and zig-zag conversion
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="371">
   <si>
     <t>date</t>
   </si>
@@ -1117,6 +1117,18 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/longest-common-prefix/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reverse words in a string</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/reverse-words-in-a-string/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zig-zag conversion</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/zigzag-conversion/</t>
   </si>
 </sst>
 </file>
@@ -3684,6 +3696,28 @@
         <v>366</v>
       </c>
     </row>
+    <row r="184" ht="14.25">
+      <c r="A184" s="1">
+        <v>46162</v>
+      </c>
+      <c r="B184" t="s">
+        <v>367</v>
+      </c>
+      <c r="C184" s="2" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="185" ht="14.25">
+      <c r="A185" s="1">
+        <v>46162</v>
+      </c>
+      <c r="B185" t="s">
+        <v>369</v>
+      </c>
+      <c r="C185" s="2" t="s">
+        <v>370</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3867,6 +3901,8 @@
     <hyperlink r:id="rId179" ref="C181"/>
     <hyperlink r:id="rId180" ref="C182"/>
     <hyperlink r:id="rId181" ref="C183"/>
+    <hyperlink r:id="rId182" ref="C184"/>
+    <hyperlink r:id="rId183" ref="C185"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: top k frequent elements
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="380">
   <si>
     <t>date</t>
   </si>
@@ -1143,10 +1143,19 @@
     <t>https://leetcode.com/problems/text-justification/</t>
   </si>
   <si>
+    <t xml:space="preserve">Striver's A-to-Z DSA Sheet+EPAM</t>
+  </si>
+  <si>
     <t xml:space="preserve">fibonacci number</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/fibonacci-number/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Top k frequent elements</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/top-k-frequent-elements/</t>
   </si>
 </sst>
 </file>
@@ -1187,7 +1196,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
@@ -1199,6 +1208,7 @@
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3759,14 +3769,32 @@
       </c>
     </row>
     <row r="188" ht="14.25">
-      <c r="A188" s="1">
+      <c r="A188" s="1"/>
+      <c r="B188" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="C188" s="2"/>
+    </row>
+    <row r="189" ht="14.25">
+      <c r="A189" s="1">
         <v>46167</v>
       </c>
-      <c r="B188" t="s">
-        <v>375</v>
-      </c>
-      <c r="C188" s="2" t="s">
+      <c r="B189" t="s">
         <v>376</v>
+      </c>
+      <c r="C189" s="2" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="190" ht="14.25">
+      <c r="A190" s="1">
+        <v>46168</v>
+      </c>
+      <c r="B190" t="s">
+        <v>378</v>
+      </c>
+      <c r="C190" s="2" t="s">
+        <v>379</v>
       </c>
     </row>
   </sheetData>
@@ -3956,7 +3984,8 @@
     <hyperlink r:id="rId183" ref="C185"/>
     <hyperlink r:id="rId184" ref="C186"/>
     <hyperlink r:id="rId185" ref="C187"/>
-    <hyperlink r:id="rId186" ref="C188"/>
+    <hyperlink r:id="rId186" ref="C189"/>
+    <hyperlink r:id="rId187" ref="C190"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: k closest points to origin
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="402">
   <si>
     <t>date</t>
   </si>
@@ -1216,6 +1216,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/kth-smallest-element-in-a-sorted-matrix/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">k closest points to origin </t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/k-closest-points-to-origin/</t>
   </si>
 </sst>
 </file>
@@ -3966,6 +3972,17 @@
         <v>399</v>
       </c>
     </row>
+    <row r="201" ht="14.25">
+      <c r="A201" s="1">
+        <v>46177</v>
+      </c>
+      <c r="B201" t="s">
+        <v>400</v>
+      </c>
+      <c r="C201" s="2" t="s">
+        <v>401</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4165,6 +4182,7 @@
     <hyperlink r:id="rId195" ref="C198"/>
     <hyperlink r:id="rId196" ref="C199"/>
     <hyperlink r:id="rId197" ref="C200"/>
+    <hyperlink r:id="rId198" ref="C201"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: reduce array size to half
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="410">
   <si>
     <t>date</t>
   </si>
@@ -1240,6 +1240,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/subset-sum-problem-1611555638/1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reduce array size to half</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/reduce-array-size-to-the-half/</t>
   </si>
 </sst>
 </file>
@@ -4034,6 +4040,17 @@
         <v>407</v>
       </c>
     </row>
+    <row r="205" ht="14.25">
+      <c r="A205" s="1">
+        <v>46179</v>
+      </c>
+      <c r="B205" t="s">
+        <v>408</v>
+      </c>
+      <c r="C205" s="2" t="s">
+        <v>409</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4237,6 +4254,7 @@
     <hyperlink r:id="rId199" ref="C202"/>
     <hyperlink r:id="rId200" ref="C203"/>
     <hyperlink r:id="rId201" ref="C204"/>
+    <hyperlink r:id="rId202" ref="C205"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: check if n and its double exist
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="414">
   <si>
     <t>date</t>
   </si>
@@ -1252,6 +1252,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/partition-equal-subset-sum/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">check if n and its double exist</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/check-if-n-and-its-double-exist/</t>
   </si>
 </sst>
 </file>
@@ -4068,6 +4074,17 @@
         <v>411</v>
       </c>
     </row>
+    <row r="207" ht="14.25">
+      <c r="A207" s="1">
+        <v>46180</v>
+      </c>
+      <c r="B207" t="s">
+        <v>412</v>
+      </c>
+      <c r="C207" s="2" t="s">
+        <v>413</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4273,6 +4290,7 @@
     <hyperlink r:id="rId201" ref="C204"/>
     <hyperlink r:id="rId202" ref="C205"/>
     <hyperlink r:id="rId203" ref="C206"/>
+    <hyperlink r:id="rId204" ref="C207"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: perfect sum problem and partition with given difference
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="420">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="422">
   <si>
     <t>date</t>
   </si>
@@ -1276,6 +1276,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/perfect-sum-problem5633/1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">partitions with given difference</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/partitions-with-given-difference/1</t>
   </si>
 </sst>
 </file>
@@ -4136,6 +4142,17 @@
         <v>419</v>
       </c>
     </row>
+    <row r="211" ht="14.25">
+      <c r="A211" s="1">
+        <v>46182</v>
+      </c>
+      <c r="B211" t="s">
+        <v>420</v>
+      </c>
+      <c r="C211" s="2" t="s">
+        <v>421</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4345,6 +4362,7 @@
     <hyperlink r:id="rId205" ref="C208"/>
     <hyperlink r:id="rId206" ref="C209"/>
     <hyperlink r:id="rId207" ref="C210"/>
+    <hyperlink r:id="rId208" ref="C211"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: remove duplicate letters
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="426">
   <si>
     <t>date</t>
   </si>
@@ -1288,6 +1288,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/minimum-cost-to-hire-k-workers/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">remove duplicate letters</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/remove-duplicate-letters/</t>
   </si>
 </sst>
 </file>
@@ -4170,6 +4176,17 @@
         <v>423</v>
       </c>
     </row>
+    <row r="213" ht="14.25">
+      <c r="A213" s="1">
+        <v>46185</v>
+      </c>
+      <c r="B213" t="s">
+        <v>424</v>
+      </c>
+      <c r="C213" s="2" t="s">
+        <v>425</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4381,6 +4398,7 @@
     <hyperlink r:id="rId207" ref="C210"/>
     <hyperlink r:id="rId208" ref="C211"/>
     <hyperlink r:id="rId209" ref="C212"/>
+    <hyperlink r:id="rId210" ref="C213"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: coin change II
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="430">
   <si>
     <t>date</t>
   </si>
@@ -1300,6 +1300,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/target-sum/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">coin change II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/coin-change-ii/</t>
   </si>
 </sst>
 </file>
@@ -4204,6 +4210,17 @@
         <v>427</v>
       </c>
     </row>
+    <row r="215" ht="14.25">
+      <c r="A215" s="1">
+        <v>46186</v>
+      </c>
+      <c r="B215" t="s">
+        <v>428</v>
+      </c>
+      <c r="C215" s="2" t="s">
+        <v>429</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4417,6 +4434,7 @@
     <hyperlink r:id="rId209" ref="C212"/>
     <hyperlink r:id="rId210" ref="C213"/>
     <hyperlink r:id="rId211" ref="C214"/>
+    <hyperlink r:id="rId212" ref="C215"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
problem: generate all binary strings without consecutive ones
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -1,22 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEE27278-72BC-44AC-AAC2-DA15AF1718A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="432">
   <si>
     <t>date</t>
   </si>
@@ -27,121 +31,121 @@
     <t>URL</t>
   </si>
   <si>
-    <t xml:space="preserve">Solution(on github repo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LCS DP</t>
+    <t>Solution(on github repo)</t>
+  </si>
+  <si>
+    <t>LCS DP</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/longest-common-subsequence/description/</t>
   </si>
   <si>
-    <t xml:space="preserve">Stock cooldown DP</t>
+    <t>Stock cooldown DP</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock-with-cooldown/</t>
   </si>
   <si>
-    <t xml:space="preserve">Stock with txn fee DP</t>
+    <t>Stock with txn fee DP</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock-with-transaction-fee/</t>
   </si>
   <si>
-    <t xml:space="preserve">Min Opns. to convert w1 to w2</t>
+    <t>Min Opns. to convert w1 to w2</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/edit-distance/</t>
   </si>
   <si>
-    <t xml:space="preserve">DP Knapsack</t>
+    <t>DP Knapsack</t>
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/0-1-knapsack-problem0945/1</t>
   </si>
   <si>
-    <t xml:space="preserve">Counting bits</t>
+    <t>Counting bits</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/counting-bits/</t>
   </si>
   <si>
-    <t xml:space="preserve">Single Number</t>
+    <t>Single Number</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/single-number/</t>
   </si>
   <si>
-    <t xml:space="preserve">Min flips to make a OR b = c</t>
+    <t>Min flips to make a OR b = c</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/minimum-flips-to-make-a-or-b-equal-to-c/description/</t>
   </si>
   <si>
-    <t xml:space="preserve">Implement Trie (Prefix Tree)</t>
+    <t>Implement Trie (Prefix Tree)</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/implement-trie-prefix-tree/</t>
   </si>
   <si>
-    <t xml:space="preserve">Search Suggestion System</t>
+    <t>Search Suggestion System</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/search-suggestions-system/description/</t>
   </si>
   <si>
-    <t xml:space="preserve">Non-Overlapping Intervals</t>
+    <t>Non-Overlapping Intervals</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/non-overlapping-intervals/</t>
   </si>
   <si>
-    <t xml:space="preserve">Min. No. of arrows for bursting ballooons</t>
+    <t>Min. No. of arrows for bursting ballooons</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/minimum-number-of-arrows-to-burst-balloons/description/</t>
   </si>
   <si>
-    <t xml:space="preserve">Daily Temperatures</t>
+    <t>Daily Temperatures</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/daily-temperatures/</t>
   </si>
   <si>
-    <t xml:space="preserve">Online Stock Span</t>
+    <t>Online Stock Span</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/online-stock-span/</t>
   </si>
   <si>
-    <t xml:space="preserve">Leetcode 150</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Merge 2 Sorted Arrays</t>
+    <t>Leetcode 150</t>
+  </si>
+  <si>
+    <t>Merge 2 Sorted Arrays</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/merge-sorted-array/</t>
   </si>
   <si>
-    <t xml:space="preserve">Climb Stairs</t>
+    <t>Climb Stairs</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/climbing-stairs/</t>
   </si>
   <si>
-    <t xml:space="preserve">House Robber</t>
+    <t>House Robber</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/house-robber/description/</t>
   </si>
   <si>
-    <t xml:space="preserve">Word Break</t>
+    <t>Word Break</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/word-break/description/</t>
   </si>
   <si>
-    <t xml:space="preserve">Coin Change</t>
+    <t>Coin Change</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/coin-change/description/</t>
@@ -159,43 +163,43 @@
     <t>https://leetcode.com/problems/triangle/</t>
   </si>
   <si>
-    <t xml:space="preserve">Min. Path Sum</t>
+    <t>Min. Path Sum</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/minimum-path-sum/</t>
   </si>
   <si>
-    <t xml:space="preserve">Unique Paths II</t>
+    <t>Unique Paths II</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/unique-paths-ii/</t>
   </si>
   <si>
-    <t xml:space="preserve">Longest Palindromic String</t>
+    <t>Longest Palindromic String</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/longest-palindromic-substring/description/</t>
   </si>
   <si>
-    <t xml:space="preserve">Check if a LL is a palindrome</t>
+    <t>Check if a LL is a palindrome</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/palindrome-linked-list/</t>
   </si>
   <si>
-    <t xml:space="preserve">Interleaving Strings</t>
+    <t>Interleaving Strings</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/interleaving-string/</t>
   </si>
   <si>
-    <t xml:space="preserve">Merge 2 Sorted LL</t>
+    <t>Merge 2 Sorted LL</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/merge-two-sorted-lists/</t>
   </si>
   <si>
-    <t xml:space="preserve">Linked List Cycle</t>
+    <t>Linked List Cycle</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/linked-list-cycle/description/</t>
@@ -207,151 +211,151 @@
     <t>https://leetcode.com/problems/remove-nth-node-from-end-of-list/</t>
   </si>
   <si>
-    <t xml:space="preserve">add 2 nos.</t>
+    <t>add 2 nos.</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/add-two-numbers/</t>
   </si>
   <si>
-    <t xml:space="preserve">edit distances</t>
+    <t>edit distances</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/edit-distance</t>
   </si>
   <si>
-    <t xml:space="preserve">best time to buy and sell stocks</t>
+    <t>best time to buy and sell stocks</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock/description/</t>
   </si>
   <si>
-    <t xml:space="preserve">best time to buy and sell stocks II</t>
+    <t>best time to buy and sell stocks II</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock-ii/</t>
   </si>
   <si>
-    <t xml:space="preserve">best time to buy and sell stocks III</t>
+    <t>best time to buy and sell stocks III</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock-iii/</t>
   </si>
   <si>
-    <t xml:space="preserve">best time to buy and sell stocks IV</t>
+    <t>best time to buy and sell stocks IV</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock-iv/</t>
   </si>
   <si>
-    <t xml:space="preserve">maximal square</t>
+    <t>maximal square</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/maximal-square/</t>
   </si>
   <si>
-    <t xml:space="preserve">no. of islands</t>
+    <t>no. of islands</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/number-of-islands/description/</t>
   </si>
   <si>
-    <t xml:space="preserve">distinct no. of islands</t>
+    <t>distinct no. of islands</t>
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/number-of-distinct-islands/1</t>
   </si>
   <si>
-    <t xml:space="preserve">surrounded regions</t>
+    <t>surrounded regions</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/surrounded-regions/</t>
   </si>
   <si>
-    <t xml:space="preserve">Contest Qn: Find Smallest Balanced Index</t>
+    <t>Contest Qn: Find Smallest Balanced Index</t>
   </si>
   <si>
     <t>https://leetcode.com/contest/weekly-contest-492/problems/find-the-smallest-balanced-index/description/</t>
   </si>
   <si>
-    <t xml:space="preserve">Min Capacity Box</t>
+    <t>Min Capacity Box</t>
   </si>
   <si>
     <t>https://leetcode.com/contest/weekly-contest-492/problems/minimum-capacity-box/description/</t>
   </si>
   <si>
-    <t xml:space="preserve">Min. opns. to sort a string</t>
+    <t>Min. opns. to sort a string</t>
   </si>
   <si>
     <t>https://leetcode.com/contest/weekly-contest-492/problems/minimum-operations-to-sort-a-string/description/</t>
   </si>
   <si>
-    <t xml:space="preserve">min cost to partition a binary string</t>
+    <t>min cost to partition a binary string</t>
   </si>
   <si>
     <t>https://leetcode.com/contest/weekly-contest-492/problems/minimum-cost-to-partition-a-binary-string/</t>
   </si>
   <si>
-    <t xml:space="preserve">clone graph</t>
+    <t>clone graph</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/clone-graph/</t>
   </si>
   <si>
-    <t xml:space="preserve">evaluate division</t>
+    <t>evaluate division</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/evaluate-division/</t>
   </si>
   <si>
-    <t xml:space="preserve">detect cycle in directed graph</t>
+    <t>detect cycle in directed graph</t>
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/detect-cycle-in-a-directed-graph/1</t>
   </si>
   <si>
-    <t xml:space="preserve">detect cycle in undirected graph</t>
+    <t>detect cycle in undirected graph</t>
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/detect-cycle-in-an-undirected-graph/1</t>
   </si>
   <si>
-    <t xml:space="preserve">topological sort</t>
+    <t>topological sort</t>
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/topological-sort/1</t>
   </si>
   <si>
-    <t xml:space="preserve">course schedule</t>
+    <t>course schedule</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/course-schedule/</t>
   </si>
   <si>
-    <t xml:space="preserve">course schedule II</t>
+    <t>course schedule II</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/course-schedule-ii/</t>
   </si>
   <si>
-    <t xml:space="preserve">Snakes and Ladders</t>
+    <t>Snakes and Ladders</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/snakes-and-ladders/</t>
   </si>
   <si>
-    <t xml:space="preserve">Minimum Genetic Mutation</t>
+    <t>Minimum Genetic Mutation</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/minimum-genetic-mutation</t>
   </si>
   <si>
-    <t xml:space="preserve">Word Ladder</t>
+    <t>Word Ladder</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/word-ladder/</t>
   </si>
   <si>
-    <t xml:space="preserve">Letter Combination of a Phone No.</t>
+    <t>Letter Combination of a Phone No.</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/letter-combinations-of-a-phone-number/</t>
@@ -369,7 +373,7 @@
     <t>https://leetcode.com/problems/permutations/</t>
   </si>
   <si>
-    <t xml:space="preserve">Combination Sum</t>
+    <t>Combination Sum</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/combination-sum/</t>
@@ -381,97 +385,97 @@
     <t>https://leetcode.com/problems/n-queens/</t>
   </si>
   <si>
-    <t xml:space="preserve">N-Queens II</t>
+    <t>N-Queens II</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/n-queens-ii/</t>
   </si>
   <si>
-    <t xml:space="preserve">Generate Paranthesis</t>
+    <t>Generate Paranthesis</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/generate-parentheses/</t>
   </si>
   <si>
-    <t xml:space="preserve">word search</t>
+    <t>word search</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/word-search/</t>
   </si>
   <si>
-    <t xml:space="preserve">maximal rectangle</t>
+    <t>maximal rectangle</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/maximal-rectangle/</t>
   </si>
   <si>
-    <t xml:space="preserve">largest rectangle in histogram</t>
+    <t>largest rectangle in histogram</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/largest-rectangle-in-histogram/</t>
   </si>
   <si>
-    <t xml:space="preserve">max depth of binary tree</t>
+    <t>max depth of binary tree</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/maximum-depth-of-binary-tree/</t>
   </si>
   <si>
-    <t xml:space="preserve">same tree</t>
+    <t>same tree</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/same-tree/</t>
   </si>
   <si>
-    <t xml:space="preserve">invert binary tree</t>
+    <t>invert binary tree</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/invert-binary-tree/</t>
   </si>
   <si>
-    <t xml:space="preserve">symmetric binary tree</t>
+    <t>symmetric binary tree</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/symmetric-tree/</t>
   </si>
   <si>
-    <t xml:space="preserve">Construct Binary Tree from inorder and preorder traversal</t>
+    <t>Construct Binary Tree from inorder and preorder traversal</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/construct-binary-tree-from-inorder-and-preorder-traversal/</t>
   </si>
   <si>
-    <t xml:space="preserve">Construct Binary Tree from inorder and postorder traversal</t>
+    <t>Construct Binary Tree from inorder and postorder traversal</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/construct-binary-tree-from-inorder-and-postorder-traversal/</t>
   </si>
   <si>
-    <t xml:space="preserve">Populating next right pointers in each node II</t>
+    <t>Populating next right pointers in each node II</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/populating-next-right-pointers-in-each-node-ii/</t>
   </si>
   <si>
-    <t xml:space="preserve">In order traversal</t>
+    <t>In order traversal</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/binary-tree-inorder-traversal/description/</t>
   </si>
   <si>
-    <t xml:space="preserve">Pre order traversal</t>
+    <t>Pre order traversal</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/binary-tree-preorder-traversal/description/</t>
   </si>
   <si>
-    <t xml:space="preserve">post order traversal</t>
+    <t>post order traversal</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/binary-tree-postorder-traversal/description/</t>
   </si>
   <si>
-    <t xml:space="preserve">flatten binary tree to linked list</t>
+    <t>flatten binary tree to linked list</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/flatten-binary-tree-to-linked-list/</t>
@@ -483,25 +487,25 @@
     <t>https://leetcode.com/problems/path-sum/</t>
   </si>
   <si>
-    <t xml:space="preserve">Path Sum II</t>
+    <t>Path Sum II</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/path-sum-ii/</t>
   </si>
   <si>
-    <t xml:space="preserve">Sum Root to Leaf numbers</t>
+    <t>Sum Root to Leaf numbers</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/sum-root-to-leaf-numbers/</t>
   </si>
   <si>
-    <t xml:space="preserve">Binary Tree Max Path Sum</t>
+    <t>Binary Tree Max Path Sum</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/binary-tree-maximum-path-sum/</t>
   </si>
   <si>
-    <t xml:space="preserve">BST Iterator</t>
+    <t>BST Iterator</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/binary-search-tree-iterator/</t>
@@ -513,67 +517,67 @@
     <t>https://leetcode.com/problems/count-complete-tree-nodes/</t>
   </si>
   <si>
-    <t xml:space="preserve">LCA of Binary Tree</t>
+    <t>LCA of Binary Tree</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-tree/</t>
   </si>
   <si>
-    <t xml:space="preserve">Binary tree right side view</t>
+    <t>Binary tree right side view</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/binary-tree-right-side-view/</t>
   </si>
   <si>
-    <t xml:space="preserve">Avg of levels in Binary Tree</t>
+    <t>Avg of levels in Binary Tree</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/average-of-levels-in-binary-tree/</t>
   </si>
   <si>
-    <t xml:space="preserve">Binary Tree level-order traversal</t>
+    <t>Binary Tree level-order traversal</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/binary-tree-level-order-traversal/</t>
   </si>
   <si>
-    <t xml:space="preserve">Binary Tree Zig-Zag traversal</t>
+    <t>Binary Tree Zig-Zag traversal</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/binary-tree-zigzag-level-order-traversal/</t>
   </si>
   <si>
-    <t xml:space="preserve">min abs diff in BST</t>
+    <t>min abs diff in BST</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/minimum-absolute-difference-in-bst/</t>
   </si>
   <si>
-    <t xml:space="preserve">kth smallest element in a BST</t>
+    <t>kth smallest element in a BST</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/kth-smallest-element-in-a-bst/</t>
   </si>
   <si>
-    <t xml:space="preserve">validate BST</t>
+    <t>validate BST</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/validate-binary-search-tree/</t>
   </si>
   <si>
-    <t xml:space="preserve">Palindrome Number</t>
+    <t>Palindrome Number</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/palindrome-number/</t>
   </si>
   <si>
-    <t xml:space="preserve">Plus One</t>
+    <t>Plus One</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/plus-one/</t>
   </si>
   <si>
-    <t xml:space="preserve">Factorial Trailing Zeroes</t>
+    <t>Factorial Trailing Zeroes</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/factorial-trailing-zeroes/</t>
@@ -591,43 +595,43 @@
     <t>https://leetcode.com/problems/powx-n/</t>
   </si>
   <si>
-    <t xml:space="preserve">Max. points on a line</t>
+    <t>Max. points on a line</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/max-points-on-a-line/</t>
   </si>
   <si>
-    <t xml:space="preserve">Add Binary</t>
+    <t>Add Binary</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/add-binary/</t>
   </si>
   <si>
-    <t xml:space="preserve">Reverse Bits</t>
+    <t>Reverse Bits</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/reverse-bits/</t>
   </si>
   <si>
-    <t xml:space="preserve">no. of set bits(Hamming Weight)</t>
+    <t>no. of set bits(Hamming Weight)</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/number-of-1-bits/</t>
   </si>
   <si>
-    <t xml:space="preserve">Single Number II</t>
+    <t>Single Number II</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/single-number-ii/</t>
   </si>
   <si>
-    <t xml:space="preserve">Bitwise and of numbers in a range</t>
+    <t>Bitwise and of numbers in a range</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/bitwise-and-of-numbers-range/</t>
   </si>
   <si>
-    <t xml:space="preserve">kth largest element in an array</t>
+    <t>kth largest element in an array</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/kth-largest-element-in-an-array/</t>
@@ -639,421 +643,421 @@
     <t>https://leetcode.com/problems/ipo/</t>
   </si>
   <si>
-    <t xml:space="preserve">max product subarray</t>
+    <t>max product subarray</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/maximum-product-subarray/</t>
   </si>
   <si>
-    <t xml:space="preserve">find k pairs with smallest sums</t>
+    <t>find k pairs with smallest sums</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/find-k-pairs-with-smallest-sums/</t>
   </si>
   <si>
-    <t xml:space="preserve">find median from data stream</t>
+    <t>find median from data stream</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/find-median-from-data-stream/</t>
   </si>
   <si>
-    <t xml:space="preserve">search insert position</t>
+    <t>search insert position</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/search-insert-position/</t>
   </si>
   <si>
-    <t xml:space="preserve">search in a 2D matrix</t>
+    <t>search in a 2D matrix</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/search-a-2d-matrix/</t>
   </si>
   <si>
-    <t xml:space="preserve">find peak element</t>
+    <t>find peak element</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/find-peak-element/</t>
   </si>
   <si>
-    <t xml:space="preserve">prefix sum range query</t>
+    <t>prefix sum range query</t>
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/prefix-sum-range-query/1</t>
   </si>
   <si>
-    <t xml:space="preserve">valid paranthesis</t>
+    <t>valid paranthesis</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/valid-parentheses/</t>
   </si>
   <si>
-    <t xml:space="preserve">next greater element</t>
+    <t>next greater element</t>
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/next-larger-element-1587115620/1</t>
   </si>
   <si>
-    <t xml:space="preserve">next greater element II</t>
+    <t>next greater element II</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/next-greater-element-ii/</t>
   </si>
   <si>
-    <t xml:space="preserve">search in sorted rotated array</t>
+    <t>search in sorted rotated array</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/search-in-rotated-sorted-array</t>
   </si>
   <si>
-    <t xml:space="preserve">find first and last position of element in sorted array</t>
+    <t>find first and last position of element in sorted array</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/find-first-and-last-position-of-element-in-sorted-array/</t>
   </si>
   <si>
-    <t xml:space="preserve">lru cache</t>
+    <t>lru cache</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/lru-cache/</t>
   </si>
   <si>
-    <t xml:space="preserve">find min. in rotated sorted array</t>
+    <t>find min. in rotated sorted array</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/find-minimum-in-rotated-sorted-array/</t>
   </si>
   <si>
-    <t xml:space="preserve">design circular queue</t>
+    <t>design circular queue</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/design-circular-queue/</t>
   </si>
   <si>
-    <t xml:space="preserve">rotate array</t>
+    <t>rotate array</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/rotate-array/</t>
   </si>
   <si>
-    <t xml:space="preserve">Median of 2 sorted arrays</t>
+    <t>Median of 2 sorted arrays</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/median-of-two-sorted-arrays/</t>
   </si>
   <si>
-    <t xml:space="preserve">maximum subarray</t>
+    <t>maximum subarray</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/maximum-subarray</t>
   </si>
   <si>
-    <t xml:space="preserve">max sum circular subarray</t>
+    <t>max sum circular subarray</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/maximum-sum-circular-subarray/</t>
   </si>
   <si>
-    <t xml:space="preserve">convert sorted array to BST</t>
+    <t>convert sorted array to BST</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/convert-sorted-array-to-binary-search-tree/</t>
   </si>
   <si>
-    <t xml:space="preserve">Sort List</t>
+    <t>Sort List</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/sort-list/</t>
   </si>
   <si>
-    <t xml:space="preserve">construct quad tree</t>
+    <t>construct quad tree</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/construct-quad-tree/</t>
   </si>
   <si>
-    <t xml:space="preserve">merge k sorted lists</t>
+    <t>merge k sorted lists</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/merge-k-sorted-lists/</t>
   </si>
   <si>
-    <t xml:space="preserve">design add and search words Data Structures</t>
+    <t>design add and search words Data Structures</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/design-add-and-search-words-data-structure/</t>
   </si>
   <si>
-    <t xml:space="preserve">word search II</t>
+    <t>word search II</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/word-search-ii/</t>
   </si>
   <si>
-    <t xml:space="preserve">copy list with random pointers</t>
+    <t>copy list with random pointers</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/copy-list-with-random-pointer/</t>
   </si>
   <si>
-    <t xml:space="preserve">reverse linked list II</t>
+    <t>reverse linked list II</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/reverse-linked-list-ii/</t>
   </si>
   <si>
-    <t xml:space="preserve">reverse nodes in k grp</t>
+    <t>reverse nodes in k grp</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/reverse-nodes-in-k-group/</t>
   </si>
   <si>
-    <t xml:space="preserve">remove duplicates from sorted list II</t>
+    <t>remove duplicates from sorted list II</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/remove-duplicates-from-sorted-list-ii/</t>
   </si>
   <si>
-    <t xml:space="preserve">rotate list</t>
+    <t>rotate list</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/rotate-list/</t>
   </si>
   <si>
-    <t xml:space="preserve">partition list</t>
+    <t>partition list</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/partition-list/</t>
   </si>
   <si>
-    <t xml:space="preserve">Simplify Path</t>
+    <t>Simplify Path</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/simplify-path/</t>
   </si>
   <si>
-    <t xml:space="preserve">min stack</t>
+    <t>min stack</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/min-stack/</t>
   </si>
   <si>
-    <t xml:space="preserve">evaluate reverse polish notation</t>
+    <t>evaluate reverse polish notation</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/evaluate-reverse-polish-notation/</t>
   </si>
   <si>
-    <t xml:space="preserve">Basic Calculator</t>
+    <t>Basic Calculator</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/basic-calculator/</t>
   </si>
   <si>
-    <t xml:space="preserve">summary ranges</t>
+    <t>summary ranges</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/summary-ranges/</t>
   </si>
   <si>
-    <t xml:space="preserve">merge intervals</t>
+    <t>merge intervals</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/merge-intervals/</t>
   </si>
   <si>
-    <t xml:space="preserve">insert intervals</t>
+    <t>insert intervals</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/insert-interval/</t>
   </si>
   <si>
-    <t xml:space="preserve">ransom note</t>
+    <t>ransom note</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/ransom-note/</t>
   </si>
   <si>
-    <t xml:space="preserve">isomorphic strings</t>
+    <t>isomorphic strings</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/isomorphic-strings/</t>
   </si>
   <si>
-    <t xml:space="preserve">word pattern</t>
+    <t>word pattern</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/word-pattern/</t>
   </si>
   <si>
-    <t xml:space="preserve">valid anagram</t>
+    <t>valid anagram</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/valid-anagram/</t>
   </si>
   <si>
-    <t xml:space="preserve">Diameter of a binary tree</t>
+    <t>Diameter of a binary tree</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/diameter-of-binary-tree/</t>
   </si>
   <si>
-    <t xml:space="preserve">Group Anagrams</t>
+    <t>Group Anagrams</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/group-anagrams/</t>
   </si>
   <si>
-    <t xml:space="preserve">Two Sum</t>
+    <t>Two Sum</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/two-sum/</t>
   </si>
   <si>
-    <t xml:space="preserve">Happy Number</t>
+    <t>Happy Number</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/happy-number/</t>
   </si>
   <si>
-    <t xml:space="preserve">contains duplicate II</t>
+    <t>contains duplicate II</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/contains-duplicate-ii/</t>
   </si>
   <si>
-    <t xml:space="preserve">longest consecutive sequence</t>
+    <t>longest consecutive sequence</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/longest-consecutive-sequence/</t>
   </si>
   <si>
-    <t xml:space="preserve">valid sudoku</t>
+    <t>valid sudoku</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/valid-sudoku/</t>
   </si>
   <si>
-    <t xml:space="preserve">spiral matrix</t>
+    <t>spiral matrix</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/spiral-matrix/</t>
   </si>
   <si>
-    <t xml:space="preserve">rotate image</t>
+    <t>rotate image</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/rotate-image/</t>
   </si>
   <si>
-    <t xml:space="preserve">set matrix zeroes</t>
+    <t>set matrix zeroes</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/set-matrix-zeroes/</t>
   </si>
   <si>
-    <t xml:space="preserve">min. size subarray sum</t>
+    <t>min. size subarray sum</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/minimum-size-subarray-sum/</t>
   </si>
   <si>
-    <t xml:space="preserve">game of life</t>
+    <t>game of life</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/game-of-life/</t>
   </si>
   <si>
-    <t xml:space="preserve">longest substring without repeating character</t>
+    <t>longest substring without repeating character</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/longest-substring-without-repeating-characters/</t>
   </si>
   <si>
-    <t xml:space="preserve">substring with concatentation of all words</t>
+    <t>substring with concatentation of all words</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/substring-with-concatenation-of-all-words/</t>
   </si>
   <si>
-    <t xml:space="preserve">min win substr.</t>
+    <t>min win substr.</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/minimum-window-substring/</t>
   </si>
   <si>
-    <t xml:space="preserve">valid palindrome</t>
+    <t>valid palindrome</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/valid-palindrome/</t>
   </si>
   <si>
-    <t xml:space="preserve">is subsequence</t>
+    <t>is subsequence</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/is-subsequence/</t>
   </si>
   <si>
-    <t xml:space="preserve">no. of matching subsequences</t>
+    <t>no. of matching subsequences</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/number-of-matching-subsequences/</t>
   </si>
   <si>
-    <t xml:space="preserve">two sum II - Input Array is Sorted</t>
+    <t>two sum II - Input Array is Sorted</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/two-sum-ii-input-array-is-sorted/</t>
   </si>
   <si>
-    <t xml:space="preserve">container with most water</t>
+    <t>container with most water</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/container-with-most-water/</t>
   </si>
   <si>
-    <t xml:space="preserve">3 sum</t>
+    <t>3 sum</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/3sum/</t>
   </si>
   <si>
-    <t xml:space="preserve">merge without extra space</t>
+    <t>merge without extra space</t>
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/merge-two-sorted-arrays-1587115620/1</t>
   </si>
   <si>
-    <t xml:space="preserve">remove element</t>
+    <t>remove element</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/remove-element/</t>
   </si>
   <si>
-    <t xml:space="preserve">remove duplicates from sorted array</t>
+    <t>remove duplicates from sorted array</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array/</t>
   </si>
   <si>
-    <t xml:space="preserve">remove duplicates from sorted array II</t>
+    <t>remove duplicates from sorted array II</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array-ii/</t>
   </si>
   <si>
-    <t xml:space="preserve">majority element</t>
+    <t>majority element</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/majority-element/</t>
   </si>
   <si>
-    <t xml:space="preserve">jump game</t>
+    <t>jump game</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/jump-game/</t>
   </si>
   <si>
-    <t xml:space="preserve">jump game II</t>
+    <t>jump game II</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/jump-game-ii/</t>
@@ -1065,19 +1069,19 @@
     <t>https://leetcode.com/problems/h-index/</t>
   </si>
   <si>
-    <t xml:space="preserve">Insert Delete Random - O(1)</t>
+    <t>Insert Delete Random - O(1)</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/insert-delete-getrandom-o1/</t>
   </si>
   <si>
-    <t xml:space="preserve">product of array except self</t>
+    <t>product of array except self</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/product-of-array-except-self/</t>
   </si>
   <si>
-    <t xml:space="preserve">Gas Station</t>
+    <t>Gas Station</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/gas-station/</t>
@@ -1089,94 +1093,94 @@
     <t>https://leetcode.com/problems/candy/</t>
   </si>
   <si>
-    <t xml:space="preserve">Trapping Rain Water</t>
+    <t>Trapping Rain Water</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/trapping-rain-water/</t>
   </si>
   <si>
-    <t xml:space="preserve">Roman to Integer</t>
+    <t>Roman to Integer</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/roman-to-integer/</t>
   </si>
   <si>
-    <t xml:space="preserve">Integer to Roman</t>
+    <t>Integer to Roman</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/integer-to-roman/</t>
   </si>
   <si>
-    <t xml:space="preserve">Length of last word</t>
+    <t>Length of last word</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/length-of-last-word/</t>
   </si>
   <si>
-    <t xml:space="preserve">longest common prefix</t>
+    <t>longest common prefix</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/longest-common-prefix/</t>
   </si>
   <si>
-    <t xml:space="preserve">reverse words in a string</t>
+    <t>reverse words in a string</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/reverse-words-in-a-string/</t>
   </si>
   <si>
-    <t xml:space="preserve">zig-zag conversion</t>
+    <t>zig-zag conversion</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/zigzag-conversion/</t>
   </si>
   <si>
-    <t xml:space="preserve">find the idx of the first occurance of the string</t>
+    <t>find the idx of the first occurance of the string</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/find-the-index-of-the-first-occurrence-in-a-string/</t>
   </si>
   <si>
-    <t xml:space="preserve">Text Justification</t>
+    <t>Text Justification</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/text-justification/</t>
   </si>
   <si>
-    <t xml:space="preserve">Striver's A-to-Z DSA Sheet+EPAM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fibonacci number</t>
+    <t>Striver's A-to-Z DSA Sheet+EPAM</t>
+  </si>
+  <si>
+    <t>fibonacci number</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/fibonacci-number/</t>
   </si>
   <si>
-    <t xml:space="preserve">Top k frequent elements</t>
+    <t>Top k frequent elements</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/top-k-frequent-elements/</t>
   </si>
   <si>
-    <t xml:space="preserve">frog jump</t>
+    <t>frog jump</t>
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/geek-jump/1</t>
   </si>
   <si>
-    <t xml:space="preserve">frog jump with k distances</t>
+    <t>frog jump with k distances</t>
   </si>
   <si>
     <t>https://takeuforward.org/plus/dsa/problems/frog-jump-with-k-distances</t>
   </si>
   <si>
-    <t xml:space="preserve">reorganize string</t>
+    <t>reorganize string</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/reorganize-string/</t>
   </si>
   <si>
-    <t xml:space="preserve">House Robber II</t>
+    <t>House Robber II</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/house-robber-ii/</t>
@@ -1188,31 +1192,31 @@
     <t>https://www.geeksforgeeks.org/problems/minimum-cost-of-ropes-1587115620/1</t>
   </si>
   <si>
-    <t xml:space="preserve">geeks training</t>
+    <t>geeks training</t>
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/geeks-training/1</t>
   </si>
   <si>
-    <t xml:space="preserve">sliding window maximum</t>
+    <t>sliding window maximum</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/sliding-window-maximum/</t>
   </si>
   <si>
-    <t xml:space="preserve">Unique Paths</t>
+    <t>Unique Paths</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/unique-paths/</t>
   </si>
   <si>
-    <t xml:space="preserve">Top k frequent words</t>
+    <t>Top k frequent words</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/top-k-frequent-words/</t>
   </si>
   <si>
-    <t xml:space="preserve">kth smallest element in a sorted matrix</t>
+    <t>kth smallest element in a sorted matrix</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/kth-smallest-element-in-a-sorted-matrix/</t>
@@ -1224,106 +1228,119 @@
     <t>https://leetcode.com/problems/k-closest-points-to-origin/</t>
   </si>
   <si>
-    <t xml:space="preserve">cherry pickup II</t>
+    <t>cherry pickup II</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/cherry-pickup-ii/</t>
   </si>
   <si>
-    <t xml:space="preserve">assign cookies</t>
+    <t>assign cookies</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/assign-cookies/</t>
   </si>
   <si>
-    <t xml:space="preserve">subset sum problem</t>
+    <t>subset sum problem</t>
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/subset-sum-problem-1611555638/1</t>
   </si>
   <si>
-    <t xml:space="preserve">reduce array size to half</t>
+    <t>reduce array size to half</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/reduce-array-size-to-the-half/</t>
   </si>
   <si>
-    <t xml:space="preserve">partition equal subset sum</t>
+    <t>partition equal subset sum</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/partition-equal-subset-sum/</t>
   </si>
   <si>
-    <t xml:space="preserve">check if n and its double exist</t>
+    <t>check if n and its double exist</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/check-if-n-and-its-double-exist/</t>
   </si>
   <si>
-    <t xml:space="preserve">min. sum partition</t>
+    <t>min. sum partition</t>
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/minimum-sum-partition3317/1</t>
   </si>
   <si>
-    <t xml:space="preserve">split a string in balanced strings</t>
+    <t>split a string in balanced strings</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/split-a-string-in-balanced-strings/</t>
   </si>
   <si>
-    <t xml:space="preserve">perfect sum problem</t>
+    <t>perfect sum problem</t>
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/perfect-sum-problem5633/1</t>
   </si>
   <si>
-    <t xml:space="preserve">partitions with given difference</t>
+    <t>partitions with given difference</t>
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/partitions-with-given-difference/1</t>
   </si>
   <si>
-    <t xml:space="preserve">minimum cost to hire k workers</t>
+    <t>minimum cost to hire k workers</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/minimum-cost-to-hire-k-workers/</t>
   </si>
   <si>
-    <t xml:space="preserve">remove duplicate letters</t>
+    <t>remove duplicate letters</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/remove-duplicate-letters/</t>
   </si>
   <si>
-    <t xml:space="preserve">target sum</t>
+    <t>target sum</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/target-sum/</t>
   </si>
   <si>
-    <t xml:space="preserve">coin change II</t>
+    <t>coin change II</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/coin-change-ii/</t>
+  </si>
+  <si>
+    <t>generate all binary strings without consecutive 1s</t>
+  </si>
+  <si>
+    <t>https://www.naukri.com/code360/problems/binary-strings-with-no-consecutive-1s_893001</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="11.000000"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
-      <sz val="11.000000"/>
+      <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1336,30 +1353,26 @@
   </fills>
   <borders count="1">
     <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1" applyFont="1"/>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1375,291 +1388,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Angsana New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Cordia New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="New Office">
       <a:dk1>
@@ -1850,20 +1580,22 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="14.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D216"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col bestFit="1" min="1" max="1" style="1" width="12.30078125"/>
-    <col bestFit="1" min="2" max="2" width="51.40234375"/>
-    <col bestFit="1" min="3" max="3" width="96.87109375"/>
-    <col bestFit="1" min="4" max="4" width="21.69140625"/>
+    <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
+    <col min="2" max="2" width="51.36328125" bestFit="1"/>
+    <col min="3" max="3" width="96.90625" bestFit="1"/>
+    <col min="4" max="4" width="21.7265625" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1877,7 +1609,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" ht="14.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>46064</v>
       </c>
@@ -1888,7 +1620,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" ht="14.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>46065</v>
       </c>
@@ -1899,7 +1631,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" ht="14.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>46066</v>
       </c>
@@ -1910,7 +1642,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" ht="14.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>46067</v>
       </c>
@@ -1921,7 +1653,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" ht="14.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>46067</v>
       </c>
@@ -1932,7 +1664,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" ht="14.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>46068</v>
       </c>
@@ -1943,7 +1675,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" ht="14.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>46069</v>
       </c>
@@ -1954,7 +1686,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" ht="14.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>46073</v>
       </c>
@@ -1965,7 +1697,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" ht="14.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>46074</v>
       </c>
@@ -1976,7 +1708,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" ht="14.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>46075</v>
       </c>
@@ -1987,7 +1719,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" ht="14.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>46076</v>
       </c>
@@ -1998,7 +1730,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" ht="14.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>46077</v>
       </c>
@@ -2009,7 +1741,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" ht="14.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>46078</v>
       </c>
@@ -2020,7 +1752,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" ht="14.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>46079</v>
       </c>
@@ -2031,12 +1763,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" ht="14.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="17" ht="14.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>46079</v>
       </c>
@@ -2047,7 +1779,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="18" ht="14.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
         <v>46080</v>
       </c>
@@ -2058,7 +1790,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" ht="14.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
         <v>46080</v>
       </c>
@@ -2069,7 +1801,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" ht="14.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>46080</v>
       </c>
@@ -2080,7 +1812,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" ht="14.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
         <v>46081</v>
       </c>
@@ -2091,7 +1823,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" ht="14.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
         <v>46081</v>
       </c>
@@ -2102,7 +1834,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" ht="14.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
         <v>46082</v>
       </c>
@@ -2113,7 +1845,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="24" ht="14.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
         <v>46082</v>
       </c>
@@ -2124,7 +1856,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="25" ht="14.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>46083</v>
       </c>
@@ -2135,7 +1867,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" ht="14.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
         <v>46083</v>
       </c>
@@ -2146,7 +1878,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="27" ht="14.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
         <v>46084</v>
       </c>
@@ -2157,7 +1889,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="28" ht="14.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
         <v>46085</v>
       </c>
@@ -2168,7 +1900,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="29" ht="14.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="1">
         <v>46085</v>
       </c>
@@ -2179,7 +1911,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="30" ht="14.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="1">
         <v>46085</v>
       </c>
@@ -2190,7 +1922,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="31" ht="14.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
         <v>46085</v>
       </c>
@@ -2201,7 +1933,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="32" ht="14.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" s="1">
         <v>46086</v>
       </c>
@@ -2212,7 +1944,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="33" ht="14.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" s="1">
         <v>46086</v>
       </c>
@@ -2223,7 +1955,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="34" ht="14.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="1">
         <v>46086</v>
       </c>
@@ -2234,40 +1966,40 @@
         <v>68</v>
       </c>
     </row>
-    <row r="35" ht="14.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" s="1">
         <v>46086</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" t="s">
         <v>69</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="36" ht="14.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" s="1">
         <v>46086</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B36" t="s">
         <v>71</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="37" ht="14.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
         <v>46087</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B37" t="s">
         <v>73</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="38" ht="14.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" s="1">
         <v>46088</v>
       </c>
@@ -2278,7 +2010,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="39" ht="14.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
         <v>46088</v>
       </c>
@@ -2289,7 +2021,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="40" ht="14.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" s="1">
         <v>46088</v>
       </c>
@@ -2300,7 +2032,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="41" ht="14.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" s="1">
         <v>46088</v>
       </c>
@@ -2311,7 +2043,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="42" ht="14.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
         <v>46089</v>
       </c>
@@ -2322,7 +2054,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="43" ht="14.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" s="1">
         <v>46089</v>
       </c>
@@ -2333,7 +2065,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="44" ht="14.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" s="1">
         <v>46089</v>
       </c>
@@ -2344,7 +2076,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="45" ht="14.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" s="1">
         <v>46089</v>
       </c>
@@ -2355,7 +2087,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="46" ht="14.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" s="1">
         <v>46089</v>
       </c>
@@ -2366,7 +2098,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="47" ht="14.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" s="1">
         <v>46090</v>
       </c>
@@ -2377,7 +2109,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="48" ht="14.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" s="1">
         <v>46090</v>
       </c>
@@ -2388,7 +2120,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="49" ht="14.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="1">
         <v>46091</v>
       </c>
@@ -2399,7 +2131,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="50" ht="14.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="1">
         <v>46091</v>
       </c>
@@ -2410,7 +2142,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="51" ht="14.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" s="1">
         <v>46091</v>
       </c>
@@ -2421,7 +2153,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="52" ht="14.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" s="1">
         <v>46092</v>
       </c>
@@ -2432,7 +2164,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="53" ht="14.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" s="1">
         <v>46093</v>
       </c>
@@ -2443,7 +2175,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="54" ht="14.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" s="1">
         <v>46094</v>
       </c>
@@ -2454,7 +2186,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="55" ht="14.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" s="1">
         <v>46095</v>
       </c>
@@ -2465,7 +2197,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="56" ht="14.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" s="1">
         <v>46096</v>
       </c>
@@ -2476,7 +2208,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="57" ht="14.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" s="1">
         <v>46096</v>
       </c>
@@ -2487,7 +2219,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="58" ht="14.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" s="1">
         <v>46097</v>
       </c>
@@ -2498,7 +2230,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="59" ht="14.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" s="1">
         <v>46097</v>
       </c>
@@ -2509,7 +2241,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="60" ht="14.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" s="1">
         <v>46098</v>
       </c>
@@ -2520,7 +2252,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="61" ht="14.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" s="1">
         <v>46098</v>
       </c>
@@ -2531,7 +2263,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="62" ht="14.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" s="1">
         <v>46099</v>
       </c>
@@ -2542,7 +2274,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="63" ht="14.25">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" s="1">
         <v>46100</v>
       </c>
@@ -2553,7 +2285,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="64" ht="14.25">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" s="1">
         <v>46100</v>
       </c>
@@ -2564,7 +2296,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="65" ht="14.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" s="1">
         <v>46100</v>
       </c>
@@ -2575,7 +2307,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="66" ht="14.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" s="1">
         <v>46101</v>
       </c>
@@ -2586,7 +2318,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="67" ht="14.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A67" s="1">
         <v>46101</v>
       </c>
@@ -2597,7 +2329,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="68" ht="14.25">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A68" s="1">
         <v>46102</v>
       </c>
@@ -2608,7 +2340,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="69" ht="14.25">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A69" s="1">
         <v>46102</v>
       </c>
@@ -2619,7 +2351,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="70" ht="14.25">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A70" s="1">
         <v>46103</v>
       </c>
@@ -2630,18 +2362,18 @@
         <v>140</v>
       </c>
     </row>
-    <row r="71" ht="14.25">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" s="1">
         <v>46103</v>
       </c>
-      <c r="B71" s="4" t="s">
+      <c r="B71" t="s">
         <v>141</v>
       </c>
       <c r="C71" s="2" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="72" ht="14.25">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" s="1">
         <v>46104</v>
       </c>
@@ -2652,7 +2384,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="73" ht="14.25">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A73" s="1">
         <v>46105</v>
       </c>
@@ -2663,7 +2395,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="74" ht="14.25">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A74" s="1">
         <v>46105</v>
       </c>
@@ -2674,7 +2406,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="75" ht="14.25">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A75" s="1">
         <v>46105</v>
       </c>
@@ -2685,7 +2417,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="76" ht="14.25">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A76" s="1">
         <v>46105</v>
       </c>
@@ -2696,7 +2428,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="77" ht="14.25">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A77" s="1">
         <v>46106</v>
       </c>
@@ -2707,7 +2439,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="78" ht="14.25">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A78" s="1">
         <v>46106</v>
       </c>
@@ -2718,7 +2450,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="79" ht="14.25">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A79" s="1">
         <v>46106</v>
       </c>
@@ -2729,7 +2461,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="80" ht="14.25">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A80" s="1">
         <v>46107</v>
       </c>
@@ -2740,7 +2472,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="81" ht="14.25">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A81" s="1">
         <v>46107</v>
       </c>
@@ -2751,7 +2483,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="82" ht="14.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A82" s="1">
         <v>46107</v>
       </c>
@@ -2762,7 +2494,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="83" ht="14.25">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A83" s="1">
         <v>46108</v>
       </c>
@@ -2773,7 +2505,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="84" ht="14.25">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A84" s="1">
         <v>46108</v>
       </c>
@@ -2784,7 +2516,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="85" ht="14.25">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A85" s="1">
         <v>46108</v>
       </c>
@@ -2795,7 +2527,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="86" ht="14.25">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A86" s="1">
         <v>46109</v>
       </c>
@@ -2806,7 +2538,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="87" ht="14.25">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A87" s="1">
         <v>46109</v>
       </c>
@@ -2817,7 +2549,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="88" ht="14.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A88" s="1">
         <v>46109</v>
       </c>
@@ -2828,7 +2560,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="89" ht="14.25">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A89" s="1">
         <v>46110</v>
       </c>
@@ -2839,7 +2571,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="90" ht="14.25">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A90" s="1">
         <v>46110</v>
       </c>
@@ -2850,7 +2582,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="91" ht="14.25">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A91" s="1">
         <v>46111</v>
       </c>
@@ -2861,7 +2593,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="92" ht="14.25">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A92" s="1">
         <v>46111</v>
       </c>
@@ -2872,7 +2604,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="93" ht="14.25">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A93" s="1">
         <v>46112</v>
       </c>
@@ -2883,7 +2615,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="94" ht="14.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A94" s="1">
         <v>46112</v>
       </c>
@@ -2894,7 +2626,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="95" ht="14.25">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A95" s="1">
         <v>46112</v>
       </c>
@@ -2905,7 +2637,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="96" ht="14.25">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A96" s="1">
         <v>46113</v>
       </c>
@@ -2916,7 +2648,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="97" ht="14.25">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A97" s="1">
         <v>46113</v>
       </c>
@@ -2927,7 +2659,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="98" ht="14.25">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A98" s="1">
         <v>46113</v>
       </c>
@@ -2938,7 +2670,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="99" ht="14.25">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A99" s="1">
         <v>46113</v>
       </c>
@@ -2949,7 +2681,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="100" ht="14.25">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A100" s="1">
         <v>46114</v>
       </c>
@@ -2960,7 +2692,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="101" ht="14.25">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A101" s="1">
         <v>46114</v>
       </c>
@@ -2971,7 +2703,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="102" ht="14.25">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A102" s="1">
         <v>46114</v>
       </c>
@@ -2982,7 +2714,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="103" ht="14.25">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A103" s="1">
         <v>46115</v>
       </c>
@@ -2993,7 +2725,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="104" ht="14.25">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A104" s="1">
         <v>46115</v>
       </c>
@@ -3004,7 +2736,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="105" ht="14.25">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A105" s="1">
         <v>46115</v>
       </c>
@@ -3015,7 +2747,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="106" ht="14.25">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A106" s="1">
         <v>46116</v>
       </c>
@@ -3026,7 +2758,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="107" ht="14.25">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A107" s="1">
         <v>46116</v>
       </c>
@@ -3037,7 +2769,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="108" ht="14.25">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A108" s="1">
         <v>46117</v>
       </c>
@@ -3048,7 +2780,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="109" ht="14.25">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A109" s="1">
         <v>46118</v>
       </c>
@@ -3059,7 +2791,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="110" ht="14.25">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A110" s="1">
         <v>46118</v>
       </c>
@@ -3070,7 +2802,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="111" ht="14.25">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A111" s="1">
         <v>46118</v>
       </c>
@@ -3081,7 +2813,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="112" ht="14.25">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A112" s="1">
         <v>46118</v>
       </c>
@@ -3092,7 +2824,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="113" ht="14.25">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A113" s="1">
         <v>46118</v>
       </c>
@@ -3103,7 +2835,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="114" ht="14.25">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A114" s="1">
         <v>46119</v>
       </c>
@@ -3114,7 +2846,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="115" ht="14.25">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A115" s="1">
         <v>46119</v>
       </c>
@@ -3125,7 +2857,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="116" ht="14.25">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A116" s="1">
         <v>46120</v>
       </c>
@@ -3136,7 +2868,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="117" ht="14.25">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A117" s="1">
         <v>46120</v>
       </c>
@@ -3147,7 +2879,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="118" ht="14.25">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A118" s="1">
         <v>46120</v>
       </c>
@@ -3158,7 +2890,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="119" ht="14.25">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A119" s="1">
         <v>46120</v>
       </c>
@@ -3169,7 +2901,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="120" ht="14.25">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A120" s="1">
         <v>46121</v>
       </c>
@@ -3180,7 +2912,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="121" ht="14.25">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A121" s="1">
         <v>46122</v>
       </c>
@@ -3191,18 +2923,18 @@
         <v>242</v>
       </c>
     </row>
-    <row r="122" ht="14.25">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A122" s="1">
         <v>46123</v>
       </c>
       <c r="B122" t="s">
         <v>243</v>
       </c>
-      <c r="C122" s="5" t="s">
+      <c r="C122" s="2" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="123" ht="14.25">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A123" s="1">
         <v>46123</v>
       </c>
@@ -3213,7 +2945,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="124" ht="14.25">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A124" s="1">
         <v>46124</v>
       </c>
@@ -3224,7 +2956,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="125" ht="14.25">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A125" s="1">
         <v>46124</v>
       </c>
@@ -3235,7 +2967,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="126" ht="14.25">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A126" s="1">
         <v>46124</v>
       </c>
@@ -3246,7 +2978,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="127" ht="14.25">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A127" s="1">
         <v>46125</v>
       </c>
@@ -3257,18 +2989,18 @@
         <v>254</v>
       </c>
     </row>
-    <row r="128" ht="14.25">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A128" s="1">
         <v>46126</v>
       </c>
       <c r="B128" t="s">
         <v>255</v>
       </c>
-      <c r="C128" s="5" t="s">
+      <c r="C128" s="2" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="129" ht="14.25">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A129" s="1">
         <v>46130</v>
       </c>
@@ -3279,7 +3011,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="130" ht="14.25">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A130" s="1">
         <v>46130</v>
       </c>
@@ -3290,7 +3022,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="131" ht="14.25">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A131" s="1">
         <v>46131</v>
       </c>
@@ -3301,7 +3033,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="132" ht="14.25">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A132" s="1">
         <v>46132</v>
       </c>
@@ -3312,7 +3044,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="133" ht="14.25">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A133" s="1">
         <v>46132</v>
       </c>
@@ -3323,7 +3055,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="134" ht="14.25">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A134" s="1">
         <v>46133</v>
       </c>
@@ -3334,7 +3066,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="135" ht="14.25">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A135" s="1">
         <v>46134</v>
       </c>
@@ -3345,7 +3077,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="136" ht="14.25">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A136" s="1">
         <v>46134</v>
       </c>
@@ -3356,7 +3088,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="137" ht="14.25">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A137" s="1">
         <v>46134</v>
       </c>
@@ -3367,7 +3099,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="138" ht="14.25">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A138" s="1">
         <v>46135</v>
       </c>
@@ -3378,7 +3110,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="139" ht="14.25">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A139" s="1">
         <v>46136</v>
       </c>
@@ -3389,7 +3121,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="140" ht="14.25">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A140" s="1">
         <v>46136</v>
       </c>
@@ -3400,7 +3132,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="141" ht="14.25">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A141" s="1">
         <v>46137</v>
       </c>
@@ -3411,7 +3143,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="142" ht="14.25">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A142" s="1">
         <v>46139</v>
       </c>
@@ -3422,7 +3154,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="143" ht="14.25">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A143" s="1">
         <v>46140</v>
       </c>
@@ -3433,7 +3165,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="144" ht="14.25">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A144" s="1">
         <v>46141</v>
       </c>
@@ -3444,7 +3176,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="145" ht="14.25">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A145" s="1">
         <v>46142</v>
       </c>
@@ -3455,7 +3187,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="146" ht="14.25">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A146" s="1">
         <v>46143</v>
       </c>
@@ -3466,7 +3198,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="147" ht="14.25">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A147" s="1">
         <v>46143</v>
       </c>
@@ -3477,7 +3209,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="148" ht="14.25">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A148" s="1">
         <v>46143</v>
       </c>
@@ -3488,7 +3220,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="149" ht="14.25">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A149" s="1">
         <v>46144</v>
       </c>
@@ -3499,7 +3231,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="150" ht="14.25">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A150" s="1">
         <v>46144</v>
       </c>
@@ -3510,7 +3242,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="151" ht="14.25">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A151" s="1">
         <v>46145</v>
       </c>
@@ -3521,7 +3253,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="152" ht="14.25">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A152" s="1">
         <v>46146</v>
       </c>
@@ -3532,7 +3264,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="153" ht="14.25">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A153" s="1">
         <v>46147</v>
       </c>
@@ -3543,7 +3275,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="154" ht="14.25">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A154" s="1">
         <v>46148</v>
       </c>
@@ -3554,7 +3286,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="155" ht="14.25">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A155" s="1">
         <v>46148</v>
       </c>
@@ -3565,7 +3297,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="156" ht="14.25">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A156" s="1">
         <v>46149</v>
       </c>
@@ -3576,7 +3308,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="157" ht="14.25">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A157" s="1">
         <v>46149</v>
       </c>
@@ -3587,7 +3319,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="158" ht="14.25">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A158" s="1">
         <v>46149</v>
       </c>
@@ -3598,7 +3330,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="159" ht="14.25">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A159" s="1">
         <v>46150</v>
       </c>
@@ -3609,7 +3341,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="160" ht="14.25">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A160" s="1">
         <v>46150</v>
       </c>
@@ -3620,7 +3352,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="161" ht="14.25">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A161" s="1">
         <v>46151</v>
       </c>
@@ -3631,7 +3363,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="162" ht="14.25">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A162" s="1">
         <v>46151</v>
       </c>
@@ -3642,7 +3374,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="163" ht="14.25">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A163" s="1">
         <v>46151</v>
       </c>
@@ -3653,7 +3385,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="164" ht="14.25">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A164" s="1">
         <v>46152</v>
       </c>
@@ -3664,7 +3396,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="165" ht="14.25">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A165" s="1">
         <v>46152</v>
       </c>
@@ -3675,7 +3407,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="166" ht="14.25">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A166" s="1">
         <v>46152</v>
       </c>
@@ -3686,7 +3418,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="167" ht="14.25">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A167" s="1">
         <v>46153</v>
       </c>
@@ -3697,7 +3429,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="168" ht="14.25">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A168" s="1">
         <v>46153</v>
       </c>
@@ -3708,7 +3440,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="169" ht="14.25">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A169" s="1">
         <v>46153</v>
       </c>
@@ -3719,7 +3451,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="170" ht="14.25">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A170" s="1">
         <v>46154</v>
       </c>
@@ -3730,18 +3462,18 @@
         <v>340</v>
       </c>
     </row>
-    <row r="171" ht="14.25">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A171" s="1">
         <v>46154</v>
       </c>
       <c r="B171" t="s">
         <v>341</v>
       </c>
-      <c r="C171" s="6" t="s">
+      <c r="C171" s="3" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="172" ht="14.25">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A172" s="1">
         <v>46155</v>
       </c>
@@ -3752,7 +3484,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="173" ht="14.25">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A173" s="1">
         <v>46155</v>
       </c>
@@ -3763,7 +3495,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="174" ht="14.25">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A174" s="1">
         <v>46157</v>
       </c>
@@ -3774,7 +3506,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="175" ht="14.25">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A175" s="1">
         <v>46157</v>
       </c>
@@ -3785,7 +3517,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="176" ht="14.25">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A176" s="1">
         <v>46158</v>
       </c>
@@ -3796,7 +3528,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="177" ht="14.25">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A177" s="1">
         <v>46158</v>
       </c>
@@ -3807,7 +3539,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="178" ht="14.25">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A178" s="1">
         <v>46159</v>
       </c>
@@ -3818,7 +3550,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="179" ht="14.25">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A179" s="1">
         <v>46159</v>
       </c>
@@ -3829,7 +3561,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="180" ht="14.25">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A180" s="1">
         <v>46160</v>
       </c>
@@ -3840,7 +3572,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="181" ht="14.25">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A181" s="1">
         <v>46160</v>
       </c>
@@ -3851,7 +3583,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="182" ht="14.25">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A182" s="1">
         <v>46161</v>
       </c>
@@ -3862,7 +3594,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="183" ht="14.25">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A183" s="1">
         <v>46161</v>
       </c>
@@ -3873,7 +3605,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="184" ht="14.25">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A184" s="1">
         <v>46162</v>
       </c>
@@ -3884,7 +3616,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="185" ht="14.25">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A185" s="1">
         <v>46162</v>
       </c>
@@ -3895,7 +3627,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="186" ht="14.25">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A186" s="1">
         <v>46163</v>
       </c>
@@ -3906,7 +3638,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="187" ht="14.25">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A187" s="1">
         <v>46165</v>
       </c>
@@ -3917,14 +3649,13 @@
         <v>374</v>
       </c>
     </row>
-    <row r="188" ht="14.25">
-      <c r="A188" s="1"/>
-      <c r="B188" s="4" t="s">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B188" t="s">
         <v>375</v>
       </c>
       <c r="C188" s="2"/>
     </row>
-    <row r="189" ht="14.25">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A189" s="1">
         <v>46167</v>
       </c>
@@ -3935,7 +3666,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="190" ht="14.25">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A190" s="1">
         <v>46168</v>
       </c>
@@ -3946,7 +3677,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="191" ht="14.25">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A191" s="1">
         <v>46168</v>
       </c>
@@ -3957,7 +3688,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="192" ht="14.25">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A192" s="1">
         <v>46169</v>
       </c>
@@ -3968,7 +3699,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="193" ht="14.25">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A193" s="1">
         <v>46170</v>
       </c>
@@ -3979,7 +3710,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="194" ht="14.25">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A194" s="1">
         <v>46171</v>
       </c>
@@ -3990,7 +3721,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="195" ht="14.25">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A195" s="1">
         <v>46172</v>
       </c>
@@ -4001,7 +3732,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="196" ht="14.25">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A196" s="1">
         <v>46172</v>
       </c>
@@ -4012,7 +3743,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="197" ht="14.25">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A197" s="1">
         <v>46173</v>
       </c>
@@ -4023,7 +3754,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="198" ht="14.25">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A198" s="1">
         <v>46173</v>
       </c>
@@ -4034,7 +3765,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="199" ht="14.25">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A199" s="1">
         <v>46174</v>
       </c>
@@ -4045,18 +3776,18 @@
         <v>397</v>
       </c>
     </row>
-    <row r="200" ht="14.25">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A200" s="1">
         <v>46175</v>
       </c>
       <c r="B200" t="s">
         <v>398</v>
       </c>
-      <c r="C200" s="5" t="s">
+      <c r="C200" s="2" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="201" ht="14.25">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A201" s="1">
         <v>46177</v>
       </c>
@@ -4067,7 +3798,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="202" ht="14.25">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A202" s="1">
         <v>46177</v>
       </c>
@@ -4078,7 +3809,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="203" ht="14.25">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A203" s="1">
         <v>46178</v>
       </c>
@@ -4089,7 +3820,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="204" ht="14.25">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A204" s="1">
         <v>46178</v>
       </c>
@@ -4100,7 +3831,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="205" ht="14.25">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A205" s="1">
         <v>46179</v>
       </c>
@@ -4111,7 +3842,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="206" ht="14.25">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A206" s="1">
         <v>46179</v>
       </c>
@@ -4122,7 +3853,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="207" ht="14.25">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A207" s="1">
         <v>46180</v>
       </c>
@@ -4133,7 +3864,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="208" ht="14.25">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A208" s="1">
         <v>46180</v>
       </c>
@@ -4144,7 +3875,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="209" ht="14.25">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A209" s="1">
         <v>46181</v>
       </c>
@@ -4155,7 +3886,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="210" ht="14.25">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A210" s="1">
         <v>46181</v>
       </c>
@@ -4166,7 +3897,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="211" ht="14.25">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A211" s="1">
         <v>46182</v>
       </c>
@@ -4177,7 +3908,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="212" ht="14.25">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A212" s="1">
         <v>46184</v>
       </c>
@@ -4188,7 +3919,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="213" ht="14.25">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A213" s="1">
         <v>46185</v>
       </c>
@@ -4199,7 +3930,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="214" ht="14.25">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A214" s="1">
         <v>46185</v>
       </c>
@@ -4210,7 +3941,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="215" ht="14.25">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A215" s="1">
         <v>46186</v>
       </c>
@@ -4221,224 +3952,234 @@
         <v>429</v>
       </c>
     </row>
+    <row r="216" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A216" s="1">
+        <v>46187</v>
+      </c>
+      <c r="B216" t="s">
+        <v>430</v>
+      </c>
+      <c r="C216" s="4" t="s">
+        <v>431</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="C2"/>
-    <hyperlink r:id="rId2" ref="C3"/>
-    <hyperlink r:id="rId3" ref="C4"/>
-    <hyperlink r:id="rId4" ref="C5"/>
-    <hyperlink r:id="rId5" ref="C6"/>
-    <hyperlink r:id="rId6" ref="C7"/>
-    <hyperlink r:id="rId7" ref="C8"/>
-    <hyperlink r:id="rId8" ref="C9"/>
-    <hyperlink r:id="rId9" ref="C10"/>
-    <hyperlink r:id="rId10" ref="C11"/>
-    <hyperlink r:id="rId11" ref="C12"/>
-    <hyperlink r:id="rId12" ref="C13"/>
-    <hyperlink r:id="rId13" ref="C14"/>
-    <hyperlink r:id="rId14" ref="C15"/>
-    <hyperlink r:id="rId15" ref="C17"/>
-    <hyperlink r:id="rId16" ref="C18"/>
-    <hyperlink r:id="rId17" ref="C19"/>
-    <hyperlink r:id="rId18" ref="C20"/>
-    <hyperlink r:id="rId19" ref="C21"/>
-    <hyperlink r:id="rId20" ref="C22"/>
-    <hyperlink r:id="rId21" ref="C23"/>
-    <hyperlink r:id="rId22" ref="C24"/>
-    <hyperlink r:id="rId23" ref="C25"/>
-    <hyperlink r:id="rId24" ref="C26"/>
-    <hyperlink r:id="rId25" ref="C27"/>
-    <hyperlink r:id="rId26" ref="C28"/>
-    <hyperlink r:id="rId27" ref="C29"/>
-    <hyperlink r:id="rId28" ref="C30"/>
-    <hyperlink r:id="rId29" ref="C31"/>
-    <hyperlink r:id="rId30" ref="C32"/>
-    <hyperlink r:id="rId31" ref="C33"/>
-    <hyperlink r:id="rId32" ref="C34"/>
-    <hyperlink r:id="rId33" ref="C35"/>
-    <hyperlink r:id="rId34" ref="C36"/>
-    <hyperlink r:id="rId35" ref="C37"/>
-    <hyperlink r:id="rId36" ref="C38"/>
-    <hyperlink r:id="rId37" ref="C39"/>
-    <hyperlink r:id="rId38" ref="C40"/>
-    <hyperlink r:id="rId39" ref="C41"/>
-    <hyperlink r:id="rId40" ref="C42"/>
-    <hyperlink r:id="rId41" ref="C43"/>
-    <hyperlink r:id="rId42" ref="C44"/>
-    <hyperlink r:id="rId43" ref="C45"/>
-    <hyperlink r:id="rId44" ref="C46"/>
-    <hyperlink r:id="rId45" ref="C47"/>
-    <hyperlink r:id="rId46" ref="C48"/>
-    <hyperlink r:id="rId47" ref="C49"/>
-    <hyperlink r:id="rId48" ref="C50"/>
-    <hyperlink r:id="rId49" ref="C51"/>
-    <hyperlink r:id="rId50" ref="C52"/>
-    <hyperlink r:id="rId51" ref="C53"/>
-    <hyperlink r:id="rId52" ref="C54"/>
-    <hyperlink r:id="rId53" ref="C55"/>
-    <hyperlink r:id="rId54" ref="C56"/>
-    <hyperlink r:id="rId55" ref="C57"/>
-    <hyperlink r:id="rId56" ref="C58"/>
-    <hyperlink r:id="rId57" ref="C59"/>
-    <hyperlink r:id="rId58" ref="C60"/>
-    <hyperlink r:id="rId59" ref="C61"/>
-    <hyperlink r:id="rId60" ref="C62"/>
-    <hyperlink r:id="rId61" ref="C63"/>
-    <hyperlink r:id="rId62" ref="C64"/>
-    <hyperlink r:id="rId63" ref="C65"/>
-    <hyperlink r:id="rId64" ref="C66"/>
-    <hyperlink r:id="rId65" ref="C67"/>
-    <hyperlink r:id="rId66" ref="C68"/>
-    <hyperlink r:id="rId67" ref="C69"/>
-    <hyperlink r:id="rId68" ref="C70"/>
-    <hyperlink r:id="rId69" ref="C71"/>
-    <hyperlink r:id="rId70" ref="C72"/>
-    <hyperlink r:id="rId71" ref="C73"/>
-    <hyperlink r:id="rId72" ref="C74"/>
-    <hyperlink r:id="rId73" ref="C75"/>
-    <hyperlink r:id="rId74" ref="C76"/>
-    <hyperlink r:id="rId75" ref="C77"/>
-    <hyperlink r:id="rId76" ref="C78"/>
-    <hyperlink r:id="rId77" ref="C79"/>
-    <hyperlink r:id="rId78" ref="C80"/>
-    <hyperlink r:id="rId79" ref="C81"/>
-    <hyperlink r:id="rId80" ref="C82"/>
-    <hyperlink r:id="rId81" ref="C83"/>
-    <hyperlink r:id="rId82" ref="C84"/>
-    <hyperlink r:id="rId83" ref="C85"/>
-    <hyperlink r:id="rId84" ref="C86"/>
-    <hyperlink r:id="rId85" ref="C87"/>
-    <hyperlink r:id="rId86" ref="C88"/>
-    <hyperlink r:id="rId87" ref="C89"/>
-    <hyperlink r:id="rId88" ref="C90"/>
-    <hyperlink r:id="rId89" ref="C91"/>
-    <hyperlink r:id="rId90" ref="C92"/>
-    <hyperlink r:id="rId91" ref="C93"/>
-    <hyperlink r:id="rId92" ref="C94"/>
-    <hyperlink r:id="rId93" ref="C95"/>
-    <hyperlink r:id="rId94" ref="C96"/>
-    <hyperlink r:id="rId95" ref="C97"/>
-    <hyperlink r:id="rId96" ref="C98"/>
-    <hyperlink r:id="rId97" ref="C99"/>
-    <hyperlink r:id="rId98" ref="C100"/>
-    <hyperlink r:id="rId99" ref="C101"/>
-    <hyperlink r:id="rId100" ref="C102"/>
-    <hyperlink r:id="rId101" ref="C103"/>
-    <hyperlink r:id="rId102" ref="C104"/>
-    <hyperlink r:id="rId103" ref="C105"/>
-    <hyperlink r:id="rId104" ref="C106"/>
-    <hyperlink r:id="rId105" ref="C107"/>
-    <hyperlink r:id="rId106" ref="C108"/>
-    <hyperlink r:id="rId107" ref="C109"/>
-    <hyperlink r:id="rId108" ref="C110"/>
-    <hyperlink r:id="rId109" ref="C111"/>
-    <hyperlink r:id="rId110" ref="C112"/>
-    <hyperlink r:id="rId111" ref="C113"/>
-    <hyperlink r:id="rId112" ref="C114"/>
-    <hyperlink r:id="rId113" ref="C115"/>
-    <hyperlink r:id="rId114" ref="C116"/>
-    <hyperlink r:id="rId115" ref="C117"/>
-    <hyperlink r:id="rId116" ref="C118"/>
-    <hyperlink r:id="rId117" ref="C119"/>
-    <hyperlink r:id="rId118" ref="C120"/>
-    <hyperlink r:id="rId119" ref="C121"/>
-    <hyperlink r:id="rId120" ref="C122"/>
-    <hyperlink r:id="rId121" ref="C123"/>
-    <hyperlink r:id="rId122" ref="C124"/>
-    <hyperlink r:id="rId123" ref="C125"/>
-    <hyperlink r:id="rId124" ref="C126"/>
-    <hyperlink r:id="rId125" ref="C127"/>
-    <hyperlink r:id="rId126" ref="C128"/>
-    <hyperlink r:id="rId127" ref="C129"/>
-    <hyperlink r:id="rId128" ref="C130"/>
-    <hyperlink r:id="rId129" ref="C131"/>
-    <hyperlink r:id="rId130" ref="C132"/>
-    <hyperlink r:id="rId131" ref="C133"/>
-    <hyperlink r:id="rId132" ref="C134"/>
-    <hyperlink r:id="rId133" ref="C135"/>
-    <hyperlink r:id="rId134" ref="C136"/>
-    <hyperlink r:id="rId135" ref="C137"/>
-    <hyperlink r:id="rId136" ref="C138"/>
-    <hyperlink r:id="rId137" ref="C139"/>
-    <hyperlink r:id="rId138" ref="C140"/>
-    <hyperlink r:id="rId139" ref="C141"/>
-    <hyperlink r:id="rId140" ref="C142"/>
-    <hyperlink r:id="rId141" ref="C143"/>
-    <hyperlink r:id="rId142" ref="C144"/>
-    <hyperlink r:id="rId143" ref="C145"/>
-    <hyperlink r:id="rId144" ref="C146"/>
-    <hyperlink r:id="rId145" ref="C147"/>
-    <hyperlink r:id="rId146" ref="C148"/>
-    <hyperlink r:id="rId147" ref="C149"/>
-    <hyperlink r:id="rId148" ref="C150"/>
-    <hyperlink r:id="rId149" ref="C151"/>
-    <hyperlink r:id="rId150" ref="C152"/>
-    <hyperlink r:id="rId151" ref="C153"/>
-    <hyperlink r:id="rId152" ref="C154"/>
-    <hyperlink r:id="rId153" ref="C155"/>
-    <hyperlink r:id="rId154" ref="C156"/>
-    <hyperlink r:id="rId155" ref="C157"/>
-    <hyperlink r:id="rId156" ref="C158"/>
-    <hyperlink r:id="rId157" ref="C159"/>
-    <hyperlink r:id="rId158" ref="C160"/>
-    <hyperlink r:id="rId159" ref="C161"/>
-    <hyperlink r:id="rId160" ref="C162"/>
-    <hyperlink r:id="rId161" ref="C163"/>
-    <hyperlink r:id="rId162" ref="C164"/>
-    <hyperlink r:id="rId163" ref="C165"/>
-    <hyperlink r:id="rId164" ref="C166"/>
-    <hyperlink r:id="rId165" ref="C167"/>
-    <hyperlink r:id="rId166" ref="C168"/>
-    <hyperlink r:id="rId167" ref="C169"/>
-    <hyperlink r:id="rId168" ref="C170"/>
-    <hyperlink r:id="rId169" ref="C171"/>
-    <hyperlink r:id="rId170" ref="C172"/>
-    <hyperlink r:id="rId171" ref="C173"/>
-    <hyperlink r:id="rId172" ref="C174"/>
-    <hyperlink r:id="rId173" ref="C175"/>
-    <hyperlink r:id="rId174" ref="C176"/>
-    <hyperlink r:id="rId175" ref="C177"/>
-    <hyperlink r:id="rId176" ref="C178"/>
-    <hyperlink r:id="rId177" ref="C179"/>
-    <hyperlink r:id="rId178" ref="C180"/>
-    <hyperlink r:id="rId179" ref="C181"/>
-    <hyperlink r:id="rId180" ref="C182"/>
-    <hyperlink r:id="rId181" ref="C183"/>
-    <hyperlink r:id="rId182" ref="C184"/>
-    <hyperlink r:id="rId183" ref="C185"/>
-    <hyperlink r:id="rId184" ref="C186"/>
-    <hyperlink r:id="rId185" ref="C187"/>
-    <hyperlink r:id="rId186" ref="C189"/>
-    <hyperlink r:id="rId187" ref="C190"/>
-    <hyperlink r:id="rId188" ref="C191"/>
-    <hyperlink r:id="rId189" ref="C192"/>
-    <hyperlink r:id="rId190" ref="C193"/>
-    <hyperlink r:id="rId191" ref="C194"/>
-    <hyperlink r:id="rId192" ref="C195"/>
-    <hyperlink r:id="rId193" ref="C196"/>
-    <hyperlink r:id="rId194" ref="C197"/>
-    <hyperlink r:id="rId195" ref="C198"/>
-    <hyperlink r:id="rId196" ref="C199"/>
-    <hyperlink r:id="rId197" ref="C200"/>
-    <hyperlink r:id="rId198" ref="C201"/>
-    <hyperlink r:id="rId199" ref="C202"/>
-    <hyperlink r:id="rId200" ref="C203"/>
-    <hyperlink r:id="rId201" ref="C204"/>
-    <hyperlink r:id="rId202" ref="C205"/>
-    <hyperlink r:id="rId203" ref="C206"/>
-    <hyperlink r:id="rId204" ref="C207"/>
-    <hyperlink r:id="rId205" ref="C208"/>
-    <hyperlink r:id="rId206" ref="C209"/>
-    <hyperlink r:id="rId207" ref="C210"/>
-    <hyperlink r:id="rId208" ref="C211"/>
-    <hyperlink r:id="rId209" ref="C212"/>
-    <hyperlink r:id="rId210" ref="C213"/>
-    <hyperlink r:id="rId211" ref="C214"/>
-    <hyperlink r:id="rId212" ref="C215"/>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="C6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="C7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="C8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="C9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="C10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="C11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="C12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="C13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="C14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="C15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="C17" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="C18" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="C19" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="C20" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="C21" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="C22" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="C23" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="C24" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="C25" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="C26" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="C27" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="C28" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="C29" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="C30" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="C31" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="C32" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="C33" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="C34" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="C35" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="C36" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="C37" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="C38" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="C39" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="C40" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="C41" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="C42" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="C43" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="C44" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="C45" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="C46" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="C47" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="C48" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="C49" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="C50" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="C51" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="C52" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="C53" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="C54" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="C55" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="C56" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="C57" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="C58" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="C59" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="C60" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="C61" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="C62" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="C63" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="C64" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="C65" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="C66" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="C67" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="C68" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="C69" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="C70" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="C71" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="C72" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="C73" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="C74" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
+    <hyperlink ref="C75" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
+    <hyperlink ref="C76" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
+    <hyperlink ref="C77" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
+    <hyperlink ref="C78" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
+    <hyperlink ref="C79" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="C80" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
+    <hyperlink ref="C81" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
+    <hyperlink ref="C82" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
+    <hyperlink ref="C83" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
+    <hyperlink ref="C84" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
+    <hyperlink ref="C85" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
+    <hyperlink ref="C86" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
+    <hyperlink ref="C87" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
+    <hyperlink ref="C88" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
+    <hyperlink ref="C89" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
+    <hyperlink ref="C90" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
+    <hyperlink ref="C91" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
+    <hyperlink ref="C92" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
+    <hyperlink ref="C93" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
+    <hyperlink ref="C94" r:id="rId92" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
+    <hyperlink ref="C95" r:id="rId93" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
+    <hyperlink ref="C96" r:id="rId94" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
+    <hyperlink ref="C97" r:id="rId95" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
+    <hyperlink ref="C98" r:id="rId96" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
+    <hyperlink ref="C99" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
+    <hyperlink ref="C100" r:id="rId98" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
+    <hyperlink ref="C101" r:id="rId99" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
+    <hyperlink ref="C102" r:id="rId100" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
+    <hyperlink ref="C103" r:id="rId101" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
+    <hyperlink ref="C104" r:id="rId102" xr:uid="{00000000-0004-0000-0000-000065000000}"/>
+    <hyperlink ref="C105" r:id="rId103" xr:uid="{00000000-0004-0000-0000-000066000000}"/>
+    <hyperlink ref="C106" r:id="rId104" xr:uid="{00000000-0004-0000-0000-000067000000}"/>
+    <hyperlink ref="C107" r:id="rId105" xr:uid="{00000000-0004-0000-0000-000068000000}"/>
+    <hyperlink ref="C108" r:id="rId106" xr:uid="{00000000-0004-0000-0000-000069000000}"/>
+    <hyperlink ref="C109" r:id="rId107" xr:uid="{00000000-0004-0000-0000-00006A000000}"/>
+    <hyperlink ref="C110" r:id="rId108" xr:uid="{00000000-0004-0000-0000-00006B000000}"/>
+    <hyperlink ref="C111" r:id="rId109" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
+    <hyperlink ref="C112" r:id="rId110" xr:uid="{00000000-0004-0000-0000-00006D000000}"/>
+    <hyperlink ref="C113" r:id="rId111" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
+    <hyperlink ref="C114" r:id="rId112" xr:uid="{00000000-0004-0000-0000-00006F000000}"/>
+    <hyperlink ref="C115" r:id="rId113" xr:uid="{00000000-0004-0000-0000-000070000000}"/>
+    <hyperlink ref="C116" r:id="rId114" xr:uid="{00000000-0004-0000-0000-000071000000}"/>
+    <hyperlink ref="C117" r:id="rId115" xr:uid="{00000000-0004-0000-0000-000072000000}"/>
+    <hyperlink ref="C118" r:id="rId116" xr:uid="{00000000-0004-0000-0000-000073000000}"/>
+    <hyperlink ref="C119" r:id="rId117" xr:uid="{00000000-0004-0000-0000-000074000000}"/>
+    <hyperlink ref="C120" r:id="rId118" xr:uid="{00000000-0004-0000-0000-000075000000}"/>
+    <hyperlink ref="C121" r:id="rId119" xr:uid="{00000000-0004-0000-0000-000076000000}"/>
+    <hyperlink ref="C122" r:id="rId120" xr:uid="{00000000-0004-0000-0000-000077000000}"/>
+    <hyperlink ref="C123" r:id="rId121" xr:uid="{00000000-0004-0000-0000-000078000000}"/>
+    <hyperlink ref="C124" r:id="rId122" xr:uid="{00000000-0004-0000-0000-000079000000}"/>
+    <hyperlink ref="C125" r:id="rId123" xr:uid="{00000000-0004-0000-0000-00007A000000}"/>
+    <hyperlink ref="C126" r:id="rId124" xr:uid="{00000000-0004-0000-0000-00007B000000}"/>
+    <hyperlink ref="C127" r:id="rId125" xr:uid="{00000000-0004-0000-0000-00007C000000}"/>
+    <hyperlink ref="C128" r:id="rId126" xr:uid="{00000000-0004-0000-0000-00007D000000}"/>
+    <hyperlink ref="C129" r:id="rId127" xr:uid="{00000000-0004-0000-0000-00007E000000}"/>
+    <hyperlink ref="C130" r:id="rId128" xr:uid="{00000000-0004-0000-0000-00007F000000}"/>
+    <hyperlink ref="C131" r:id="rId129" xr:uid="{00000000-0004-0000-0000-000080000000}"/>
+    <hyperlink ref="C132" r:id="rId130" xr:uid="{00000000-0004-0000-0000-000081000000}"/>
+    <hyperlink ref="C133" r:id="rId131" xr:uid="{00000000-0004-0000-0000-000082000000}"/>
+    <hyperlink ref="C134" r:id="rId132" xr:uid="{00000000-0004-0000-0000-000083000000}"/>
+    <hyperlink ref="C135" r:id="rId133" xr:uid="{00000000-0004-0000-0000-000084000000}"/>
+    <hyperlink ref="C136" r:id="rId134" xr:uid="{00000000-0004-0000-0000-000085000000}"/>
+    <hyperlink ref="C137" r:id="rId135" xr:uid="{00000000-0004-0000-0000-000086000000}"/>
+    <hyperlink ref="C138" r:id="rId136" xr:uid="{00000000-0004-0000-0000-000087000000}"/>
+    <hyperlink ref="C139" r:id="rId137" xr:uid="{00000000-0004-0000-0000-000088000000}"/>
+    <hyperlink ref="C140" r:id="rId138" xr:uid="{00000000-0004-0000-0000-000089000000}"/>
+    <hyperlink ref="C141" r:id="rId139" xr:uid="{00000000-0004-0000-0000-00008A000000}"/>
+    <hyperlink ref="C142" r:id="rId140" xr:uid="{00000000-0004-0000-0000-00008B000000}"/>
+    <hyperlink ref="C143" r:id="rId141" xr:uid="{00000000-0004-0000-0000-00008C000000}"/>
+    <hyperlink ref="C144" r:id="rId142" xr:uid="{00000000-0004-0000-0000-00008D000000}"/>
+    <hyperlink ref="C145" r:id="rId143" xr:uid="{00000000-0004-0000-0000-00008E000000}"/>
+    <hyperlink ref="C146" r:id="rId144" xr:uid="{00000000-0004-0000-0000-00008F000000}"/>
+    <hyperlink ref="C147" r:id="rId145" xr:uid="{00000000-0004-0000-0000-000090000000}"/>
+    <hyperlink ref="C148" r:id="rId146" xr:uid="{00000000-0004-0000-0000-000091000000}"/>
+    <hyperlink ref="C149" r:id="rId147" xr:uid="{00000000-0004-0000-0000-000092000000}"/>
+    <hyperlink ref="C150" r:id="rId148" xr:uid="{00000000-0004-0000-0000-000093000000}"/>
+    <hyperlink ref="C151" r:id="rId149" xr:uid="{00000000-0004-0000-0000-000094000000}"/>
+    <hyperlink ref="C152" r:id="rId150" xr:uid="{00000000-0004-0000-0000-000095000000}"/>
+    <hyperlink ref="C153" r:id="rId151" xr:uid="{00000000-0004-0000-0000-000096000000}"/>
+    <hyperlink ref="C154" r:id="rId152" xr:uid="{00000000-0004-0000-0000-000097000000}"/>
+    <hyperlink ref="C155" r:id="rId153" xr:uid="{00000000-0004-0000-0000-000098000000}"/>
+    <hyperlink ref="C156" r:id="rId154" xr:uid="{00000000-0004-0000-0000-000099000000}"/>
+    <hyperlink ref="C157" r:id="rId155" xr:uid="{00000000-0004-0000-0000-00009A000000}"/>
+    <hyperlink ref="C158" r:id="rId156" xr:uid="{00000000-0004-0000-0000-00009B000000}"/>
+    <hyperlink ref="C159" r:id="rId157" xr:uid="{00000000-0004-0000-0000-00009C000000}"/>
+    <hyperlink ref="C160" r:id="rId158" xr:uid="{00000000-0004-0000-0000-00009D000000}"/>
+    <hyperlink ref="C161" r:id="rId159" xr:uid="{00000000-0004-0000-0000-00009E000000}"/>
+    <hyperlink ref="C162" r:id="rId160" xr:uid="{00000000-0004-0000-0000-00009F000000}"/>
+    <hyperlink ref="C163" r:id="rId161" xr:uid="{00000000-0004-0000-0000-0000A0000000}"/>
+    <hyperlink ref="C164" r:id="rId162" xr:uid="{00000000-0004-0000-0000-0000A1000000}"/>
+    <hyperlink ref="C165" r:id="rId163" xr:uid="{00000000-0004-0000-0000-0000A2000000}"/>
+    <hyperlink ref="C166" r:id="rId164" xr:uid="{00000000-0004-0000-0000-0000A3000000}"/>
+    <hyperlink ref="C167" r:id="rId165" xr:uid="{00000000-0004-0000-0000-0000A4000000}"/>
+    <hyperlink ref="C168" r:id="rId166" xr:uid="{00000000-0004-0000-0000-0000A5000000}"/>
+    <hyperlink ref="C169" r:id="rId167" xr:uid="{00000000-0004-0000-0000-0000A6000000}"/>
+    <hyperlink ref="C170" r:id="rId168" xr:uid="{00000000-0004-0000-0000-0000A7000000}"/>
+    <hyperlink ref="C171" r:id="rId169" xr:uid="{00000000-0004-0000-0000-0000A8000000}"/>
+    <hyperlink ref="C172" r:id="rId170" xr:uid="{00000000-0004-0000-0000-0000A9000000}"/>
+    <hyperlink ref="C173" r:id="rId171" xr:uid="{00000000-0004-0000-0000-0000AA000000}"/>
+    <hyperlink ref="C174" r:id="rId172" xr:uid="{00000000-0004-0000-0000-0000AB000000}"/>
+    <hyperlink ref="C175" r:id="rId173" xr:uid="{00000000-0004-0000-0000-0000AC000000}"/>
+    <hyperlink ref="C176" r:id="rId174" xr:uid="{00000000-0004-0000-0000-0000AD000000}"/>
+    <hyperlink ref="C177" r:id="rId175" xr:uid="{00000000-0004-0000-0000-0000AE000000}"/>
+    <hyperlink ref="C178" r:id="rId176" xr:uid="{00000000-0004-0000-0000-0000AF000000}"/>
+    <hyperlink ref="C179" r:id="rId177" xr:uid="{00000000-0004-0000-0000-0000B0000000}"/>
+    <hyperlink ref="C180" r:id="rId178" xr:uid="{00000000-0004-0000-0000-0000B1000000}"/>
+    <hyperlink ref="C181" r:id="rId179" xr:uid="{00000000-0004-0000-0000-0000B2000000}"/>
+    <hyperlink ref="C182" r:id="rId180" xr:uid="{00000000-0004-0000-0000-0000B3000000}"/>
+    <hyperlink ref="C183" r:id="rId181" xr:uid="{00000000-0004-0000-0000-0000B4000000}"/>
+    <hyperlink ref="C184" r:id="rId182" xr:uid="{00000000-0004-0000-0000-0000B5000000}"/>
+    <hyperlink ref="C185" r:id="rId183" xr:uid="{00000000-0004-0000-0000-0000B6000000}"/>
+    <hyperlink ref="C186" r:id="rId184" xr:uid="{00000000-0004-0000-0000-0000B7000000}"/>
+    <hyperlink ref="C187" r:id="rId185" xr:uid="{00000000-0004-0000-0000-0000B8000000}"/>
+    <hyperlink ref="C189" r:id="rId186" xr:uid="{00000000-0004-0000-0000-0000B9000000}"/>
+    <hyperlink ref="C190" r:id="rId187" xr:uid="{00000000-0004-0000-0000-0000BA000000}"/>
+    <hyperlink ref="C191" r:id="rId188" xr:uid="{00000000-0004-0000-0000-0000BB000000}"/>
+    <hyperlink ref="C192" r:id="rId189" xr:uid="{00000000-0004-0000-0000-0000BC000000}"/>
+    <hyperlink ref="C193" r:id="rId190" xr:uid="{00000000-0004-0000-0000-0000BD000000}"/>
+    <hyperlink ref="C194" r:id="rId191" xr:uid="{00000000-0004-0000-0000-0000BE000000}"/>
+    <hyperlink ref="C195" r:id="rId192" xr:uid="{00000000-0004-0000-0000-0000BF000000}"/>
+    <hyperlink ref="C196" r:id="rId193" xr:uid="{00000000-0004-0000-0000-0000C0000000}"/>
+    <hyperlink ref="C197" r:id="rId194" xr:uid="{00000000-0004-0000-0000-0000C1000000}"/>
+    <hyperlink ref="C198" r:id="rId195" xr:uid="{00000000-0004-0000-0000-0000C2000000}"/>
+    <hyperlink ref="C199" r:id="rId196" xr:uid="{00000000-0004-0000-0000-0000C3000000}"/>
+    <hyperlink ref="C200" r:id="rId197" xr:uid="{00000000-0004-0000-0000-0000C4000000}"/>
+    <hyperlink ref="C201" r:id="rId198" xr:uid="{00000000-0004-0000-0000-0000C5000000}"/>
+    <hyperlink ref="C202" r:id="rId199" xr:uid="{00000000-0004-0000-0000-0000C6000000}"/>
+    <hyperlink ref="C203" r:id="rId200" xr:uid="{00000000-0004-0000-0000-0000C7000000}"/>
+    <hyperlink ref="C204" r:id="rId201" xr:uid="{00000000-0004-0000-0000-0000C8000000}"/>
+    <hyperlink ref="C205" r:id="rId202" xr:uid="{00000000-0004-0000-0000-0000C9000000}"/>
+    <hyperlink ref="C206" r:id="rId203" xr:uid="{00000000-0004-0000-0000-0000CA000000}"/>
+    <hyperlink ref="C207" r:id="rId204" xr:uid="{00000000-0004-0000-0000-0000CB000000}"/>
+    <hyperlink ref="C208" r:id="rId205" xr:uid="{00000000-0004-0000-0000-0000CC000000}"/>
+    <hyperlink ref="C209" r:id="rId206" xr:uid="{00000000-0004-0000-0000-0000CD000000}"/>
+    <hyperlink ref="C210" r:id="rId207" xr:uid="{00000000-0004-0000-0000-0000CE000000}"/>
+    <hyperlink ref="C211" r:id="rId208" xr:uid="{00000000-0004-0000-0000-0000CF000000}"/>
+    <hyperlink ref="C212" r:id="rId209" xr:uid="{00000000-0004-0000-0000-0000D0000000}"/>
+    <hyperlink ref="C213" r:id="rId210" xr:uid="{00000000-0004-0000-0000-0000D1000000}"/>
+    <hyperlink ref="C214" r:id="rId211" xr:uid="{00000000-0004-0000-0000-0000D2000000}"/>
+    <hyperlink ref="C215" r:id="rId212" xr:uid="{00000000-0004-0000-0000-0000D3000000}"/>
+    <hyperlink ref="C216" r:id="rId213" xr:uid="{95DADF51-0029-47AE-8E17-84E67D521B48}"/>
   </hyperlinks>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="0" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId214"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: print longest common subsequence
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D76FD90-D778-49A7-A7AF-18EB26D67066}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11BEB9C4-9028-4CDB-B987-69F4B3DF9379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="440">
   <si>
     <t>date</t>
   </si>
@@ -1334,6 +1334,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/letter-case-permutation/</t>
+  </si>
+  <si>
+    <t>Print LCS</t>
+  </si>
+  <si>
+    <t>https://www.naukri.com/code360/problems/print-longest-common-subsequence_8416383</t>
   </si>
 </sst>
 </file>
@@ -1604,7 +1610,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D219"/>
+  <dimension ref="A1:D220"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4012,6 +4018,17 @@
       </c>
       <c r="C219" s="4" t="s">
         <v>437</v>
+      </c>
+    </row>
+    <row r="220" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A220" s="1">
+        <v>46189</v>
+      </c>
+      <c r="B220" t="s">
+        <v>438</v>
+      </c>
+      <c r="C220" s="4" t="s">
+        <v>439</v>
       </c>
     </row>
   </sheetData>
@@ -4232,8 +4249,9 @@
     <hyperlink ref="C217" r:id="rId214" xr:uid="{B43A0CB5-E214-4BC9-8A56-6FD8D2AA8D99}"/>
     <hyperlink ref="C218" r:id="rId215" xr:uid="{E551B356-82F4-4DEE-A9B6-4CAC836DBBCF}"/>
     <hyperlink ref="C219" r:id="rId216" xr:uid="{7A3C069D-6D65-4B6A-900E-33694EA1BBFA}"/>
+    <hyperlink ref="C220" r:id="rId217" xr:uid="{2EA4DE40-0D59-4EAD-92A5-E1D46D0BEE9C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId217"/>
+  <pageSetup orientation="portrait" r:id="rId218"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problems: word search, longest common substring and max. length of repeated subarray
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11BEB9C4-9028-4CDB-B987-69F4B3DF9379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B67503-A513-4C7E-936E-D51959199C5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="444">
   <si>
     <t>date</t>
   </si>
@@ -1340,6 +1340,18 @@
   </si>
   <si>
     <t>https://www.naukri.com/code360/problems/print-longest-common-subsequence_8416383</t>
+  </si>
+  <si>
+    <t>longest common substring</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/longest-common-substring1452/1</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/maximum-length-of-repeated-subarray/</t>
+  </si>
+  <si>
+    <t>max. length of repeated subarray</t>
   </si>
 </sst>
 </file>
@@ -1610,7 +1622,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D220"/>
+  <dimension ref="A1:D222"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4029,6 +4041,28 @@
       </c>
       <c r="C220" s="4" t="s">
         <v>439</v>
+      </c>
+    </row>
+    <row r="221" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A221" s="1">
+        <v>46190</v>
+      </c>
+      <c r="B221" t="s">
+        <v>440</v>
+      </c>
+      <c r="C221" s="4" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="222" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A222" s="1">
+        <v>46190</v>
+      </c>
+      <c r="B222" t="s">
+        <v>443</v>
+      </c>
+      <c r="C222" s="4" t="s">
+        <v>442</v>
       </c>
     </row>
   </sheetData>
@@ -4250,8 +4284,10 @@
     <hyperlink ref="C218" r:id="rId215" xr:uid="{E551B356-82F4-4DEE-A9B6-4CAC836DBBCF}"/>
     <hyperlink ref="C219" r:id="rId216" xr:uid="{7A3C069D-6D65-4B6A-900E-33694EA1BBFA}"/>
     <hyperlink ref="C220" r:id="rId217" xr:uid="{2EA4DE40-0D59-4EAD-92A5-E1D46D0BEE9C}"/>
+    <hyperlink ref="C221" r:id="rId218" xr:uid="{105DCDB4-957A-406A-9D90-380F57E707C1}"/>
+    <hyperlink ref="C222" r:id="rId219" xr:uid="{76B8EA9C-8138-4EC3-9D55-58B047142A44}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId218"/>
+  <pageSetup orientation="portrait" r:id="rId220"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problems: expression add operators and min. insertions to make a string palindrome
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FAEFE29-4E73-434A-B26C-2422C0A53D19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AAA13ED-2EDF-4050-909D-BAA292A9AF0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="454">
   <si>
     <t>date</t>
   </si>
@@ -1370,6 +1370,18 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/combination-sum-iii</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min insertions required to make a string palindrome </t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-insertion-steps-to-make-a-string-palindrome/</t>
+  </si>
+  <si>
+    <t>expression add operators</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/expression-add-operators/</t>
   </si>
 </sst>
 </file>
@@ -1640,7 +1652,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D225"/>
+  <dimension ref="A1:D227"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4114,6 +4126,28 @@
       </c>
       <c r="C225" s="4" t="s">
         <v>449</v>
+      </c>
+    </row>
+    <row r="226" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A226" s="1">
+        <v>46192</v>
+      </c>
+      <c r="B226" t="s">
+        <v>452</v>
+      </c>
+      <c r="C226" s="4" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="227" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A227" s="1">
+        <v>46192</v>
+      </c>
+      <c r="B227" t="s">
+        <v>450</v>
+      </c>
+      <c r="C227" s="4" t="s">
+        <v>451</v>
       </c>
     </row>
   </sheetData>
@@ -4340,8 +4374,10 @@
     <hyperlink ref="C223" r:id="rId220" xr:uid="{599031F7-CBC5-47CC-8203-C2B0C0939432}"/>
     <hyperlink ref="C224" r:id="rId221" xr:uid="{2520CA58-6164-40D0-A139-89878326E026}"/>
     <hyperlink ref="C225" r:id="rId222" xr:uid="{74DCE01A-E90F-4335-BC09-6944BD888142}"/>
+    <hyperlink ref="C227" r:id="rId223" xr:uid="{F129DF05-12AE-4F8B-B901-10D9824B64C3}"/>
+    <hyperlink ref="C226" r:id="rId224" xr:uid="{1738018E-5280-4EBF-B0E5-1880B2CBBC97}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId223"/>
+  <pageSetup orientation="portrait" r:id="rId225"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: shortest common super sequence
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4349746E-A776-4CD3-9D96-8C6B01DB3482}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44E5009B-FACE-40DA-9712-BB859181C236}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="458">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="460">
   <si>
     <t>date</t>
   </si>
@@ -1394,6 +1394,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/find-the-highest-altitude/</t>
+  </si>
+  <si>
+    <t>shortest common subsequence</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/shortest-common-supersequence/</t>
   </si>
 </sst>
 </file>
@@ -1664,7 +1670,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D229"/>
+  <dimension ref="A1:D230"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4182,6 +4188,17 @@
       </c>
       <c r="C229" s="4" t="s">
         <v>457</v>
+      </c>
+    </row>
+    <row r="230" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A230" s="1">
+        <v>46193</v>
+      </c>
+      <c r="B230" t="s">
+        <v>458</v>
+      </c>
+      <c r="C230" s="4" t="s">
+        <v>459</v>
       </c>
     </row>
   </sheetData>
@@ -4412,8 +4429,9 @@
     <hyperlink ref="C226" r:id="rId224" xr:uid="{1738018E-5280-4EBF-B0E5-1880B2CBBC97}"/>
     <hyperlink ref="C228" r:id="rId225" xr:uid="{6299FE99-DC4E-4BA9-A436-CA76F577B238}"/>
     <hyperlink ref="C229" r:id="rId226" xr:uid="{CED6339E-BA64-40EC-809F-8F6683BD2FFB}"/>
+    <hyperlink ref="C230" r:id="rId227" xr:uid="{18B3952D-D773-4220-83A8-5DFCBE47BE6B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId227"/>
+  <pageSetup orientation="portrait" r:id="rId228"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: largest divisible subset
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7057770A-0D13-45B9-8512-68BC4780DDA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E991288-1FC5-48D7-8DBF-5BBFFA897A47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="468">
   <si>
     <t>date</t>
   </si>
@@ -1418,6 +1418,12 @@
   </si>
   <si>
     <t>printing LIS</t>
+  </si>
+  <si>
+    <t>largest divisble subset</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/largest-divisible-subset/</t>
   </si>
 </sst>
 </file>
@@ -1688,7 +1694,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D233"/>
+  <dimension ref="A1:D234"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4250,6 +4256,17 @@
       </c>
       <c r="C233" s="4" t="s">
         <v>464</v>
+      </c>
+    </row>
+    <row r="234" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A234" s="1">
+        <v>46200</v>
+      </c>
+      <c r="B234" t="s">
+        <v>466</v>
+      </c>
+      <c r="C234" s="4" t="s">
+        <v>467</v>
       </c>
     </row>
   </sheetData>
@@ -4484,8 +4501,9 @@
     <hyperlink ref="C231" r:id="rId228" xr:uid="{B5E70D10-CDC3-4746-8E93-23E7DE722147}"/>
     <hyperlink ref="C232" r:id="rId229" xr:uid="{7874E577-FFBF-45D8-811A-8A6780B02C8C}"/>
     <hyperlink ref="C233" r:id="rId230" xr:uid="{1AB23B31-A231-42A7-92AD-E1E7D40A5E67}"/>
+    <hyperlink ref="C234" r:id="rId231" xr:uid="{D41A7E5E-D532-4BBD-9F17-A2984DAE138E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId231"/>
+  <pageSetup orientation="portrait" r:id="rId232"/>
 </worksheet>
 </file>
</xml_diff>